<commit_message>
fix: align timetable workload and localization
</commit_message>
<xml_diff>
--- a/outputs/stage-7/school-data-import-template.xlsx
+++ b/outputs/stage-7/school-data-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rf74cb03946814ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="R1652ca5b039b4d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rcfde8092f6bf4da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="R673540739133431b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
         <x:v>academic_period</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>{"id":"term_1_2026","label":"Synthetic Term 1","start_date":"2026-09-01","end_date":"2026-12-24","days":[{"id":"mon","label":"Monday","ordinal":1},{"id":"tue","label":"Tuesday","ordinal":2},{"id":"wed","label":"Wednesday","ordinal":3},{"id":"thu","label":"Thursday","ordinal":4},{"id":"fri","label":"Friday","ordinal":5}],"periods":[{"id":"p1","label":"Period 1","ordinal":1,"start_time":"08:00","end_time":"08:45"},{"id":"p2","label":"Period 2","ordinal":2,"start_time":"08:55","end_time":"09:40"},{"id":"p3","label":"Period 3","ordinal":3,"start_time":"10:00","end_time":"10:45"},{"id":"p4","label":"Period 4","ordinal":4,"start_time":"11:05","end_time":"11:50"},{"id":"p5","label":"Period 5","ordinal":5,"start_time":"12:00","end_time":"12:45"},{"id":"p6","label":"Period 6","ordinal":6,"start_time":"12:55","end_time":"13:40"}],"shifts":[{"id":"morning","label":"Morning shift","period_ids":["p1","p2","p3","p4","p5","p6"]}]}</x:v>
+        <x:v>{"id":"term_1_2026","label":"Synthetic Term 1","start_date":"2026-09-01","end_date":"2026-12-24","days":[{"id":"mon","label":"Monday","ordinal":1},{"id":"tue","label":"Tuesday","ordinal":2},{"id":"wed","label":"Wednesday","ordinal":3},{"id":"thu","label":"Thursday","ordinal":4},{"id":"fri","label":"Friday","ordinal":5}],"periods":[{"id":"p1","label":"Period 1","ordinal":1,"start_time":"08:00","end_time":"08:45"},{"id":"p2","label":"Period 2","ordinal":2,"start_time":"08:55","end_time":"09:40"},{"id":"p3","label":"Period 3","ordinal":3,"start_time":"10:00","end_time":"10:45"},{"id":"p4","label":"Period 4","ordinal":4,"start_time":"11:05","end_time":"11:50"},{"id":"p5","label":"Period 5","ordinal":5,"start_time":"12:00","end_time":"12:45"},{"id":"p6","label":"Period 6","ordinal":6,"start_time":"12:55","end_time":"13:40"},{"id":"p7","label":"Period 7","ordinal":7,"start_time":"13:50","end_time":"14:35"}],"shifts":[{"id":"morning","label":"Morning shift","period_ids":["p1","p2","p3","p4","p5","p6","p7"]}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
@@ -558,7 +558,7 @@
         <x:v>policies</x:v>
       </x:c>
       <x:c r="B16" s="15" t="str">
-        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_7a"},"maximum":6},{"resource":{"type":"class","id":"class_8a"},"maximum":6},{"resource":{"type":"teacher","id":"t_math"},"maximum":6}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_7a"},"target":6},{"participant":{"type":"class","id":"class_8a"},"target":6}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P2","weight":4},{"constraint_id":"SC-003","priority":"P1","weight":8},{"constraint_id":"SC-004","priority":"P2","weight":3},{"constraint_id":"SC-005","priority":"P2","weight":4}]}</x:v>
+        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_7a"},"maximum":7},{"resource":{"type":"class","id":"class_8a"},"maximum":7},{"resource":{"type":"teacher","id":"t_math"},"maximum":6}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_7a"},"target":6},{"participant":{"type":"class","id":"class_8a"},"target":6}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P2","weight":4},{"constraint_id":"SC-003","priority":"P1","weight":8},{"constraint_id":"SC-004","priority":"P2","weight":3},{"constraint_id":"SC-005","priority":"P2","weight":4}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">

</xml_diff>

<commit_message>
fix: generate complete school timetables
</commit_message>
<xml_diff>
--- a/outputs/stage-7/school-data-import-template.xlsx
+++ b/outputs/stage-7/school-data-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rcfde8092f6bf4da0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="R673540739133431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rab0dae508ed54259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="Rb8d2c5a50ffe46ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -462,7 +462,7 @@
         <x:v>school</x:v>
       </x:c>
       <x:c r="B4" s="15" t="str">
-        <x:v>{"id":"demo_school","label":"Synthetic Demonstration School","timezone":"Europe/Minsk"}</x:v>
+        <x:v>{"id":"demo_school","label":"Representative Demonstration School","timezone":"Europe/Minsk"}</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
@@ -470,7 +470,7 @@
         <x:v>academic_period</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>{"id":"term_1_2026","label":"Synthetic Term 1","start_date":"2026-09-01","end_date":"2026-12-24","days":[{"id":"mon","label":"Monday","ordinal":1},{"id":"tue","label":"Tuesday","ordinal":2},{"id":"wed","label":"Wednesday","ordinal":3},{"id":"thu","label":"Thursday","ordinal":4},{"id":"fri","label":"Friday","ordinal":5}],"periods":[{"id":"p1","label":"Period 1","ordinal":1,"start_time":"08:00","end_time":"08:45"},{"id":"p2","label":"Period 2","ordinal":2,"start_time":"08:55","end_time":"09:40"},{"id":"p3","label":"Period 3","ordinal":3,"start_time":"10:00","end_time":"10:45"},{"id":"p4","label":"Period 4","ordinal":4,"start_time":"11:05","end_time":"11:50"},{"id":"p5","label":"Period 5","ordinal":5,"start_time":"12:00","end_time":"12:45"},{"id":"p6","label":"Period 6","ordinal":6,"start_time":"12:55","end_time":"13:40"},{"id":"p7","label":"Period 7","ordinal":7,"start_time":"13:50","end_time":"14:35"}],"shifts":[{"id":"morning","label":"Morning shift","period_ids":["p1","p2","p3","p4","p5","p6","p7"]}]}</x:v>
+        <x:v>{"id":"term_1_2026","label":"Demonstration Term 1","start_date":"2026-09-01","end_date":"2026-12-24","days":[{"id":"mon","label":"Monday","ordinal":1},{"id":"tue","label":"Tuesday","ordinal":2},{"id":"wed","label":"Wednesday","ordinal":3},{"id":"thu","label":"Thursday","ordinal":4},{"id":"fri","label":"Friday","ordinal":5}],"periods":[{"id":"p1","label":"Period 1","ordinal":1,"start_time":"08:00","end_time":"08:45"},{"id":"p2","label":"Period 2","ordinal":2,"start_time":"08:55","end_time":"09:40"},{"id":"p3","label":"Period 3","ordinal":3,"start_time":"10:00","end_time":"10:45"},{"id":"p4","label":"Period 4","ordinal":4,"start_time":"11:05","end_time":"11:50"},{"id":"p5","label":"Period 5","ordinal":5,"start_time":"12:00","end_time":"12:45"},{"id":"p6","label":"Period 6","ordinal":6,"start_time":"12:55","end_time":"13:40"},{"id":"p7","label":"Period 7","ordinal":7,"start_time":"13:50","end_time":"14:35"}],"shifts":[{"id":"morning","label":"Morning shift","period_ids":["p1","p2","p3","p4","p5","p6","p7"]}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
@@ -478,7 +478,7 @@
         <x:v>subjects</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
-        <x:v>[{"id":"mathematics","label":"Mathematics","default_workload":3},{"id":"physics","label":"Physics","default_workload":3},{"id":"chemistry","label":"Chemistry","default_workload":3},{"id":"english","label":"English","default_workload":2},{"id":"history","label":"History","default_workload":2},{"id":"physical_education","label":"Physical Education","default_workload":1},{"id":"advisory","label":"Advisory","default_workload":1}]</x:v>
+        <x:v>[{"id":"mathematics","label":"Mathematics","default_workload":3},{"id":"russian_language","label":"Russian Language","default_workload":3},{"id":"russian_literature","label":"Russian Literature","default_workload":2},{"id":"belarusian_language","label":"Belarusian Language","default_workload":3},{"id":"belarusian_literature","label":"Belarusian Literature","default_workload":2},{"id":"english","label":"English","default_workload":2},{"id":"physical_education","label":"Physical Education","default_workload":1},{"id":"technology","label":"Technology","default_workload":1},{"id":"informatics","label":"Informatics","default_workload":2},{"id":"art","label":"Art","default_workload":1},{"id":"human_and_world","label":"Human and the World","default_workload":1},{"id":"life_safety","label":"Life Safety","default_workload":1},{"id":"biology","label":"Biology","default_workload":3},{"id":"geography","label":"Geography","default_workload":2},{"id":"history_belarus","label":"History of Belarus","default_workload":2},{"id":"world_history","label":"World History","default_workload":2},{"id":"physics","label":"Physics","default_workload":3},{"id":"chemistry","label":"Chemistry","default_workload":3},{"id":"social_studies","label":"Social Studies","default_workload":2},{"id":"technical_drawing","label":"Technical Drawing","default_workload":2},{"id":"astronomy","label":"Astronomy","default_workload":3},{"id":"defense_medical","label":"Defense and Medical Training","default_workload":1}]</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
@@ -486,7 +486,7 @@
         <x:v>teachers</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>[{"id":"t_math","label":"Teacher T-Math","qualified_subject_ids":["mathematics"]},{"id":"t_science","label":"Teacher T-Science","qualified_subject_ids":["physics","chemistry"]},{"id":"t_english_a","label":"Teacher T-English-A","qualified_subject_ids":["english"]},{"id":"t_english_b","label":"Teacher T-English-B","qualified_subject_ids":["english"]},{"id":"t_history","label":"Teacher T-History","qualified_subject_ids":["history","advisory"]},{"id":"t_pe","label":"Teacher T-PE","qualified_subject_ids":["physical_education"]}]</x:v>
+        <x:v>[{"id":"t_math","label":"Teacher T-5A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_5b","label":"Teacher T-5B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_5v","label":"Teacher T-5V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6a","label":"Teacher T-6A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6b","label":"Teacher T-6B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6v","label":"Teacher T-6V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7a","label":"Teacher T-7A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7b","label":"Teacher T-7B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7v","label":"Teacher T-7V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_8a","label":"Teacher T-8A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_8b","label":"Teacher T-8B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9a","label":"Teacher T-9A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9b","label":"Teacher T-9B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9v","label":"Teacher T-9V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_10a","label":"Teacher T-10A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_10b","label":"Teacher T-10B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_11a","label":"Teacher T-11A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_11b","label":"Teacher T-11B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_science","label":"Teacher T-Science","qualified_subject_ids":["physics","chemistry"]},{"id":"t_english_a","label":"Teacher T-English-A","qualified_subject_ids":["english"]},{"id":"t_english_b","label":"Teacher T-English-B","qualified_subject_ids":["english"]},{"id":"t_history","label":"Teacher T-History","qualified_subject_ids":["art"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
@@ -494,7 +494,7 @@
         <x:v>classrooms</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>[{"id":"room_101","label":"Room 101","capacity":30,"capabilities":["general"]},{"id":"room_102","label":"Room 102","capacity":30,"capabilities":["general"]},{"id":"science_lab","label":"Science Laboratory","capacity":24,"capabilities":["general","physics_lab","chemistry_lab"]},{"id":"gym","label":"Gymnasium","capacity":60,"capabilities":["sports"]},{"id":"hall","label":"Assembly Hall","capacity":60,"capabilities":["assembly"]}]</x:v>
+        <x:v>[{"id":"room_5a","label":"Room 5A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5b","label":"Room 5B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5v","label":"Room 5V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6a","label":"Room 6A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6b","label":"Room 6B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6v","label":"Room 6V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7a","label":"Room 7A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7b","label":"Room 7B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7v","label":"Room 7V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8a","label":"Room 8A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8b","label":"Room 8B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9a","label":"Room 9A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9b","label":"Room 9B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9v","label":"Room 9V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10a","label":"Room 10A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10b","label":"Room 10B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11a","label":"Room 11A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11b","label":"Room 11B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"science_lab","label":"Science Laboratory","capacity":30,"capabilities":["general","physics_lab","chemistry_lab"]},{"id":"hall","label":"Assembly Hall","capacity":60,"capabilities":["assembly"]},{"id":"language_room_a","label":"Language Room A","capacity":30,"capabilities":["general"]},{"id":"language_room_b","label":"Language Room B","capacity":30,"capabilities":["general"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="45" customHeight="1">
@@ -502,7 +502,7 @@
         <x:v>classes</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>[{"id":"class_7a","label":"Class 7A","grade":7,"student_count":24,"shift_id":"morning"},{"id":"class_8a","label":"Class 8A","grade":8,"student_count":22,"shift_id":"morning"}]</x:v>
+        <x:v>[{"id":"class_5a","label":"Class 5A","grade":5,"student_count":26,"shift_id":"morning"},{"id":"class_5b","label":"Class 5B","grade":5,"student_count":27,"shift_id":"morning"},{"id":"class_5v","label":"Class 5V","grade":5,"student_count":27,"shift_id":"morning"},{"id":"class_6a","label":"Class 6A","grade":6,"student_count":27,"shift_id":"morning"},{"id":"class_6b","label":"Class 6B","grade":6,"student_count":28,"shift_id":"morning"},{"id":"class_6v","label":"Class 6V","grade":6,"student_count":28,"shift_id":"morning"},{"id":"class_7a","label":"Class 7A","grade":7,"student_count":28,"shift_id":"morning"},{"id":"class_7b","label":"Class 7B","grade":7,"student_count":24,"shift_id":"morning"},{"id":"class_7v","label":"Class 7V","grade":7,"student_count":24,"shift_id":"morning"},{"id":"class_8a","label":"Class 8A","grade":8,"student_count":24,"shift_id":"morning"},{"id":"class_8b","label":"Class 8B","grade":8,"student_count":25,"shift_id":"morning"},{"id":"class_9a","label":"Class 9A","grade":9,"student_count":25,"shift_id":"morning"},{"id":"class_9b","label":"Class 9B","grade":9,"student_count":26,"shift_id":"morning"},{"id":"class_9v","label":"Class 9V","grade":9,"student_count":26,"shift_id":"morning"},{"id":"class_10a","label":"Class 10A","grade":10,"student_count":26,"shift_id":"morning"},{"id":"class_10b","label":"Class 10B","grade":10,"student_count":27,"shift_id":"morning"},{"id":"class_11a","label":"Class 11A","grade":11,"student_count":27,"shift_id":"morning"},{"id":"class_11b","label":"Class 11B","grade":11,"student_count":28,"shift_id":"morning"}]</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="45" customHeight="1">
@@ -518,7 +518,7 @@
         <x:v>groups</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>[{"id":"group_7a_en_1","label":"Class 7A English Group 1","class_id":"class_7a","partition_id":"partition_7a_english","student_count":12},{"id":"group_7a_en_2","label":"Class 7A English Group 2","class_id":"class_7a","partition_id":"partition_7a_english","student_count":12}]</x:v>
+        <x:v>[{"id":"group_7a_en_1","label":"Class 7A English Group 1","class_id":"class_7a","partition_id":"partition_7a_english","student_count":14},{"id":"group_7a_en_2","label":"Class 7A English Group 2","class_id":"class_7a","partition_id":"partition_7a_english","student_count":14}]</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
@@ -534,7 +534,7 @@
         <x:v>curriculum_requirements</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
-        <x:v>[{"id":"req_7a_math","participant":{"type":"class","id":"class_7a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_7a_physics","participant":{"type":"class","id":"class_7a"},"subject_id":"physics","eligible_teacher_ids":["t_science"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["physics_lab"],"allowed_classroom_ids":["science_lab"]},{"id":"req_7a_en_1","participant":{"type":"group","id":"group_7a_en_1"},"subject_id":"english","eligible_teacher_ids":["t_english_a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_7a_en_2","participant":{"type":"group","id":"group_7a_en_2"},"subject_id":"english","eligible_teacher_ids":["t_english_b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_7a_history","participant":{"type":"class","id":"class_7a"},"subject_id":"history","eligible_teacher_ids":["t_history"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_7a_pe","participant":{"type":"class","id":"class_7a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["sports"],"allowed_classroom_ids":["gym"]},{"id":"req_8a_math","participant":{"type":"class","id":"class_8a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_8a_chemistry","participant":{"type":"class","id":"class_8a"},"subject_id":"chemistry","eligible_teacher_ids":["t_science"],"weekly_lessons":2,"block_length":2,"required_room_capabilities":["chemistry_lab"],"allowed_classroom_ids":["science_lab"]},{"id":"req_8a_english","participant":{"type":"class","id":"class_8a"},"subject_id":"english","eligible_teacher_ids":["t_english_a","t_english_b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_8a_history","participant":{"type":"class","id":"class_8a"},"subject_id":"history","eligible_teacher_ids":["t_history"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":[]},{"id":"req_8a_pe","participant":{"type":"class","id":"class_8a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["sports"],"allowed_classroom_ids":["gym"]},{"id":"req_joint_advisory","participant":{"type":"cohort","id":"cohort_7a_8a_advisory"},"subject_id":"advisory","eligible_teacher_ids":["t_history"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["assembly"],"allowed_classroom_ids":["hall"]}]</x:v>
+        <x:v>[{"id":"req_5a_mathematics","participant":{"type":"class","id":"class_5a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_language","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_english","participant":{"type":"class","id":"class_5a"},"subject_id":"english","eligible_teacher_ids":["t_math"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_physical_education","participant":{"type":"class","id":"class_5a"},"subject_id":"physical_education","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_technology","participant":{"type":"class","id":"class_5a"},"subject_id":"technology","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_art","participant":{"type":"class","id":"class_5a"},"subject_id":"art","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_human_and_world","participant":{"type":"class","id":"class_5a"},"subject_id":"human_and_world","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_life_safety","participant":{"type":"class","id":"class_5a"},"subject_id":"life_safety","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_world_history","participant":{"type":"class","id":"class_5a"},"subject_id":"world_history","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5b_mathematics","participant":{"type":"class","id":"class_5b"},"subject_id":"mathematics","eligible_teacher_ids":["t_5b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_language","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_english","participant":{"type":"class","id":"class_5b"},"subject_id":"english","eligible_teacher_ids":["t_5b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_physical_education","participant":{"type":"class","id":"class_5b"},"subject_id":"physical_education","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_technology","participant":{"type":"class","id":"class_5b"},"subject_id":"technology","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_art","participant":{"type":"class","id":"class_5b"},"subject_id":"art","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_human_and_world","participant":{"type":"class","id":"class_5b"},"subject_id":"human_and_world","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_life_safety","participant":{"type":"class","id":"class_5b"},"subject_id":"life_safety","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_world_history","participant":{"type":"class","id":"class_5b"},"subject_id":"world_history","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5v_mathematics","participant":{"type":"class","id":"class_5v"},"subject_id":"mathematics","eligible_teacher_ids":["t_5v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_language","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_english","participant":{"type":"class","id":"class_5v"},"subject_id":"english","eligible_teacher_ids":["t_5v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_physical_education","participant":{"type":"class","id":"class_5v"},"subject_id":"physical_education","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_technology","participant":{"type":"class","id":"class_5v"},"subject_id":"technology","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_art","participant":{"type":"class","id":"class_5v"},"subject_id":"art","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_human_and_world","participant":{"type":"class","id":"class_5v"},"subject_id":"human_and_world","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_life_safety","participant":{"type":"class","id":"class_5v"},"subject_id":"life_safety","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_world_history","participant":{"type":"class","id":"class_5v"},"subject_id":"world_history","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_6a_mathematics","participant":{"type":"class","id":"class_6a"},"subject_id":"mathematics","eligible_teacher_ids":["t_6a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_language","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_english","participant":{"type":"class","id":"class_6a"},"subject_id":"english","eligible_teacher_ids":["t_6a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_physical_education","participant":{"type":"class","id":"class_6a"},"subject_id":"physical_education","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_technology","participant":{"type":"class","id":"class_6a"},"subject_id":"technology","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_informatics","participant":{"type":"class","id":"class_6a"},"subject_id":"informatics","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_art","participant":{"type":"class","id":"class_6a"},"subject_id":"art","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_biology","participant":{"type":"class","id":"class_6a"},"subject_id":"biology","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_geography","participant":{"type":"class","id":"class_6a"},"subject_id":"geography","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_history_belarus","participant":{"type":"class","id":"class_6a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_world_history","participant":{"type":"class","id":"class_6a"},"subject_id":"world_history","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6b_mathematics","participant":{"type":"class","id":"class_6b"},"subject_id":"mathematics","eligible_teacher_ids":["t_6b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_language","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_english","participant":{"type":"class","id":"class_6b"},"subject_id":"english","eligible_teacher_ids":["t_6b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_physical_education","participant":{"type":"class","id":"class_6b"},"subject_id":"physical_education","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_technology","participant":{"type":"class","id":"class_6b"},"subject_id":"technology","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_informatics","participant":{"type":"class","id":"class_6b"},"subject_id":"informatics","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_art","participant":{"type":"class","id":"class_6b"},"subject_id":"art","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_biology","participant":{"type":"class","id":"class_6b"},"subject_id":"biology","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_geography","participant":{"type":"class","id":"class_6b"},"subject_id":"geography","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_history_belarus","participant":{"type":"class","id":"class_6b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_world_history","participant":{"type":"class","id":"class_6b"},"subject_id":"world_history","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6v_mathematics","participant":{"type":"class","id":"class_6v"},"subject_id":"mathematics","eligible_teacher_ids":["t_6v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_language","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_english","participant":{"type":"class","id":"class_6v"},"subject_id":"english","eligible_teacher_ids":["t_6v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_physical_education","participant":{"type":"class","id":"class_6v"},"subject_id":"physical_education","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_technology","participant":{"type":"class","id":"class_6v"},"subject_id":"technology","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_informatics","participant":{"type":"class","id":"class_6v"},"subject_id":"informatics","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_art","participant":{"type":"class","id":"class_6v"},"subject_id":"art","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_biology","participant":{"type":"class","id":"class_6v"},"subject_id":"biology","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_geography","participant":{"type":"class","id":"class_6v"},"subject_id":"geography","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_history_belarus","participant":{"type":"class","id":"class_6v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_world_history","participant":{"type":"class","id":"class_6v"},"subject_id":"world_history","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_7a_math","participant":{"type":"class","id":"class_7a"},"subject_id":"mathematics","eligible_teacher_ids":["t_7a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_language","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_en_1","participant":{"type":"class","id":"class_7a"},"subject_id":"english","eligible_teacher_ids":["t_7a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physical_education","participant":{"type":"class","id":"class_7a"},"subject_id":"physical_education","eligible_teacher_ids":["t_7a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_technology","participant":{"type":"class","id":"class_7a"},"subject_id":"technology","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_informatics","participant":{"type":"class","id":"class_7a"},"subject_id":"informatics","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_joint_advisory","participant":{"type":"class","id":"class_7a"},"subject_id":"art","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_biology","participant":{"type":"class","id":"class_7a"},"subject_id":"biology","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_geography","participant":{"type":"class","id":"class_7a"},"subject_id":"geography","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_history_belarus","participant":{"type":"class","id":"class_7a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_world_history","participant":{"type":"class","id":"class_7a"},"subject_id":"world_history","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physics","participant":{"type":"class","id":"class_7a"},"subject_id":"physics","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_chemistry","participant":{"type":"class","id":"class_7a"},"subject_id":"chemistry","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7b_mathematics","participant":{"type":"class","id":"class_7b"},"subject_id":"mathematics","eligible_teacher_ids":["t_7b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_language","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_english","participant":{"type":"class","id":"class_7b"},"subject_id":"english","eligible_teacher_ids":["t_7b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physical_education","participant":{"type":"class","id":"class_7b"},"subject_id":"physical_education","eligible_teacher_ids":["t_7b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_technology","participant":{"type":"class","id":"class_7b"},"subject_id":"technology","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_informatics","participant":{"type":"class","id":"class_7b"},"subject_id":"informatics","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_art","participant":{"type":"class","id":"class_7b"},"subject_id":"art","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_biology","participant":{"type":"class","id":"class_7b"},"subject_id":"biology","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_geography","participant":{"type":"class","id":"class_7b"},"subject_id":"geography","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_history_belarus","participant":{"type":"class","id":"class_7b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_world_history","participant":{"type":"class","id":"class_7b"},"subject_id":"world_history","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physics","participant":{"type":"class","id":"class_7b"},"subject_id":"physics","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_chemistry","participant":{"type":"class","id":"class_7b"},"subject_id":"chemistry","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7v_mathematics","participant":{"type":"class","id":"class_7v"},"subject_id":"mathematics","eligible_teacher_ids":["t_7v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_language","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_english","participant":{"type":"class","id":"class_7v"},"subject_id":"english","eligible_teacher_ids":["t_7v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physical_education","participant":{"type":"class","id":"class_7v"},"subject_id":"physical_education","eligible_teacher_ids":["t_7v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_technology","participant":{"type":"class","id":"class_7v"},"subject_id":"technology","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_informatics","participant":{"type":"class","id":"class_7v"},"subject_id":"informatics","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_art","participant":{"type":"class","id":"class_7v"},"subject_id":"art","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_biology","participant":{"type":"class","id":"class_7v"},"subject_id":"biology","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_geography","participant":{"type":"class","id":"class_7v"},"subject_id":"geography","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_history_belarus","participant":{"type":"class","id":"class_7v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_world_history","participant":{"type":"class","id":"class_7v"},"subject_id":"world_history","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physics","participant":{"type":"class","id":"class_7v"},"subject_id":"physics","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_chemistry","participant":{"type":"class","id":"class_7v"},"subject_id":"chemistry","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_8a_mathematics","participant":{"type":"class","id":"class_8a"},"subject_id":"mathematics","eligible_teacher_ids":["t_8a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_language","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_english","participant":{"type":"class","id":"class_8a"},"subject_id":"english","eligible_teacher_ids":["t_8a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physical_education","participant":{"type":"class","id":"class_8a"},"subject_id":"physical_education","eligible_teacher_ids":["t_8a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_technology","participant":{"type":"class","id":"class_8a"},"subject_id":"technology","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_informatics","participant":{"type":"class","id":"class_8a"},"subject_id":"informatics","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_art","participant":{"type":"class","id":"class_8a"},"subject_id":"art","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_biology","participant":{"type":"class","id":"class_8a"},"subject_id":"biology","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_geography","participant":{"type":"class","id":"class_8a"},"subject_id":"geography","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_history_belarus","participant":{"type":"class","id":"class_8a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_world_history","participant":{"type":"class","id":"class_8a"},"subject_id":"world_history","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physics","participant":{"type":"class","id":"class_8a"},"subject_id":"physics","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_chemistry","participant":{"type":"class","id":"class_8a"},"subject_id":"chemistry","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":2,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8b_mathematics","participant":{"type":"class","id":"class_8b"},"subject_id":"mathematics","eligible_teacher_ids":["t_8b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_language","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_english","participant":{"type":"class","id":"class_8b"},"subject_id":"english","eligible_teacher_ids":["t_8b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physical_education","participant":{"type":"class","id":"class_8b"},"subject_id":"physical_education","eligible_teacher_ids":["t_8b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_technology","participant":{"type":"class","id":"class_8b"},"subject_id":"technology","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_informatics","participant":{"type":"class","id":"class_8b"},"subject_id":"informatics","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_art","participant":{"type":"class","id":"class_8b"},"subject_id":"art","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_biology","participant":{"type":"class","id":"class_8b"},"subject_id":"biology","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_geography","participant":{"type":"class","id":"class_8b"},"subject_id":"geography","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_history_belarus","participant":{"type":"class","id":"class_8b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_world_history","participant":{"type":"class","id":"class_8b"},"subject_id":"world_history","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physics","participant":{"type":"class","id":"class_8b"},"subject_id":"physics","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_chemistry","participant":{"type":"class","id":"class_8b"},"subject_id":"chemistry","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_9a_mathematics","participant":{"type":"class","id":"class_9a"},"subject_id":"mathematics","eligible_teacher_ids":["t_9a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_language","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_english","participant":{"type":"class","id":"class_9a"},"subject_id":"english","eligible_teacher_ids":["t_9a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physical_education","participant":{"type":"class","id":"class_9a"},"subject_id":"physical_education","eligible_teacher_ids":["t_9a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_technology","participant":{"type":"class","id":"class_9a"},"subject_id":"technology","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_informatics","participant":{"type":"class","id":"class_9a"},"subject_id":"informatics","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_biology","participant":{"type":"class","id":"class_9a"},"subject_id":"biology","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_geography","participant":{"type":"class","id":"class_9a"},"subject_id":"geography","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_history_belarus","participant":{"type":"class","id":"class_9a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_world_history","participant":{"type":"class","id":"class_9a"},"subject_id":"world_history","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physics","participant":{"type":"class","id":"class_9a"},"subject_id":"physics","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_chemistry","participant":{"type":"class","id":"class_9a"},"subject_id":"chemistry","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_social_studies","participant":{"type":"class","id":"class_9a"},"subject_id":"social_studies","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9b_mathematics","participant":{"type":"class","id":"class_9b"},"subject_id":"mathematics","eligible_teacher_ids":["t_9b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_language","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_english","participant":{"type":"class","id":"class_9b"},"subject_id":"english","eligible_teacher_ids":["t_9b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physical_education","participant":{"type":"class","id":"class_9b"},"subject_id":"physical_education","eligible_teacher_ids":["t_9b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_technology","participant":{"type":"class","id":"class_9b"},"subject_id":"technology","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_informatics","participant":{"type":"class","id":"class_9b"},"subject_id":"informatics","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_biology","participant":{"type":"class","id":"class_9b"},"subject_id":"biology","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_geography","participant":{"type":"class","id":"class_9b"},"subject_id":"geography","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_history_belarus","participant":{"type":"class","id":"class_9b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_world_history","participant":{"type":"class","id":"class_9b"},"subject_id":"world_history","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physics","participant":{"type":"class","id":"class_9b"},"subject_id":"physics","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_chemistry","participant":{"type":"class","id":"class_9b"},"subject_id":"chemistry","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_social_studies","participant":{"type":"class","id":"class_9b"},"subject_id":"social_studies","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9v_mathematics","participant":{"type":"class","id":"class_9v"},"subject_id":"mathematics","eligible_teacher_ids":["t_9v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_language","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_english","participant":{"type":"class","id":"class_9v"},"subject_id":"english","eligible_teacher_ids":["t_9v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physical_education","participant":{"type":"class","id":"class_9v"},"subject_id":"physical_education","eligible_teacher_ids":["t_9v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_technology","participant":{"type":"class","id":"class_9v"},"subject_id":"technology","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_informatics","participant":{"type":"class","id":"class_9v"},"subject_id":"informatics","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_biology","participant":{"type":"class","id":"class_9v"},"subject_id":"biology","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_geography","participant":{"type":"class","id":"class_9v"},"subject_id":"geography","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_history_belarus","participant":{"type":"class","id":"class_9v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_world_history","participant":{"type":"class","id":"class_9v"},"subject_id":"world_history","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physics","participant":{"type":"class","id":"class_9v"},"subject_id":"physics","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_chemistry","participant":{"type":"class","id":"class_9v"},"subject_id":"chemistry","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_social_studies","participant":{"type":"class","id":"class_9v"},"subject_id":"social_studies","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_10a_mathematics","participant":{"type":"class","id":"class_10a"},"subject_id":"mathematics","eligible_teacher_ids":["t_10a"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physics","participant":{"type":"class","id":"class_10a"},"subject_id":"physics","eligible_teacher_ids":["t_10a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_chemistry","participant":{"type":"class","id":"class_10a"},"subject_id":"chemistry","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_biology","participant":{"type":"class","id":"class_10a"},"subject_id":"biology","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_language","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_english","participant":{"type":"class","id":"class_10a"},"subject_id":"english","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physical_education","participant":{"type":"class","id":"class_10a"},"subject_id":"physical_education","eligible_teacher_ids":["t_10a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_informatics","participant":{"type":"class","id":"class_10a"},"subject_id":"informatics","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_geography","participant":{"type":"class","id":"class_10a"},"subject_id":"geography","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_history_belarus","participant":{"type":"class","id":"class_10a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_social_studies","participant":{"type":"class","id":"class_10a"},"subject_id":"social_studies","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_technical_drawing","participant":{"type":"class","id":"class_10a"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_defense_medical","participant":{"type":"class","id":"class_10a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10b_mathematics","participant":{"type":"class","id":"class_10b"},"subject_id":"mathematics","eligible_teacher_ids":["t_10b"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physics","participant":{"type":"class","id":"class_10b"},"subject_id":"physics","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_chemistry","participant":{"type":"class","id":"class_10b"},"subject_id":"chemistry","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_biology","participant":{"type":"class","id":"class_10b"},"subject_id":"biology","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_language","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_english","participant":{"type":"class","id":"class_10b"},"subject_id":"english","eligible_teacher_ids":["t_10b"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physical_education","participant":{"type":"class","id":"class_10b"},"subject_id":"physical_education","eligible_teacher_ids":["t_10b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_informatics","participant":{"type":"class","id":"class_10b"},"subject_id":"informatics","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_geography","participant":{"type":"class","id":"class_10b"},"subject_id":"geography","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_history_belarus","participant":{"type":"class","id":"class_10b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_social_studies","participant":{"type":"class","id":"class_10b"},"subject_id":"social_studies","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_technical_drawing","participant":{"type":"class","id":"class_10b"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_defense_medical","participant":{"type":"class","id":"class_10b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_11a_mathematics","participant":{"type":"class","id":"class_11a"},"subject_id":"mathematics","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physics","participant":{"type":"class","id":"class_11a"},"subject_id":"physics","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_chemistry","participant":{"type":"class","id":"class_11a"},"subject_id":"chemistry","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_biology","participant":{"type":"class","id":"class_11a"},"subject_id":"biology","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_language","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_english","participant":{"type":"class","id":"class_11a"},"subject_id":"english","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physical_education","participant":{"type":"class","id":"class_11a"},"subject_id":"physical_education","eligible_teacher_ids":["t_11a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_informatics","participant":{"type":"class","id":"class_11a"},"subject_id":"informatics","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_geography","participant":{"type":"class","id":"class_11a"},"subject_id":"geography","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_history_belarus","participant":{"type":"class","id":"class_11a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_social_studies","participant":{"type":"class","id":"class_11a"},"subject_id":"social_studies","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_astronomy","participant":{"type":"class","id":"class_11a"},"subject_id":"astronomy","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_defense_medical","participant":{"type":"class","id":"class_11a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11b_mathematics","participant":{"type":"class","id":"class_11b"},"subject_id":"mathematics","eligible_teacher_ids":["t_11b"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physics","participant":{"type":"class","id":"class_11b"},"subject_id":"physics","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_chemistry","participant":{"type":"class","id":"class_11b"},"subject_id":"chemistry","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_biology","participant":{"type":"class","id":"class_11b"},"subject_id":"biology","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_language","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_english","participant":{"type":"class","id":"class_11b"},"subject_id":"english","eligible_teacher_ids":["t_11b"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physical_education","participant":{"type":"class","id":"class_11b"},"subject_id":"physical_education","eligible_teacher_ids":["t_11b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_informatics","participant":{"type":"class","id":"class_11b"},"subject_id":"informatics","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_geography","participant":{"type":"class","id":"class_11b"},"subject_id":"geography","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_history_belarus","participant":{"type":"class","id":"class_11b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_social_studies","participant":{"type":"class","id":"class_11b"},"subject_id":"social_studies","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_astronomy","participant":{"type":"class","id":"class_11b"},"subject_id":"astronomy","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_defense_medical","participant":{"type":"class","id":"class_11b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
@@ -542,7 +542,7 @@
         <x:v>resource_availability</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>[{"resource":{"type":"teacher","id":"t_math"},"unavailable_slots":[{"day_id":"tue","period_id":"p1"}],"preferred_slots":[{"day_id":"mon","period_id":"p2"}]},{"resource":{"type":"classroom","id":"science_lab"},"unavailable_slots":[{"day_id":"fri","period_id":"p6"}],"preferred_slots":[]}]</x:v>
+        <x:v>[{"resource":{"type":"class","id":"class_5a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9v"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"teacher","id":"t_math"},"unavailable_slots":[],"preferred_slots":[]},{"resource":{"type":"teacher","id":"t_7a"},"unavailable_slots":[],"preferred_slots":[]},{"resource":{"type":"classroom","id":"science_lab"},"unavailable_slots":[{"day_id":"fri","period_id":"p6"}],"preferred_slots":[]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
@@ -550,7 +550,7 @@
         <x:v>fixed_lessons</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>[{"id":"fixed_joint_advisory","requirement_id":"req_joint_advisory","occurrence_index":0,"slot":{"day_id":"mon","period_id":"p1"},"teacher_id":"t_history","classroom_id":"hall"}]</x:v>
+        <x:v>[{"id":"fixed_joint_advisory","requirement_id":"req_joint_advisory","occurrence_index":0,"slot":{"day_id":"mon","period_id":"p1"},"teacher_id":"t_7a","classroom_id":"room_7a"}]</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
@@ -558,7 +558,7 @@
         <x:v>policies</x:v>
       </x:c>
       <x:c r="B16" s="15" t="str">
-        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_7a"},"maximum":7},{"resource":{"type":"class","id":"class_8a"},"maximum":7},{"resource":{"type":"teacher","id":"t_math"},"maximum":6}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_7a"},"target":6},{"participant":{"type":"class","id":"class_8a"},"target":6}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P2","weight":4},{"constraint_id":"SC-003","priority":"P1","weight":8},{"constraint_id":"SC-004","priority":"P2","weight":3},{"constraint_id":"SC-005","priority":"P2","weight":4}]}</x:v>
+        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_5a"},"maximum":6},{"resource":{"type":"teacher","id":"t_math"},"maximum":6},{"resource":{"type":"class","id":"class_5b"},"maximum":6},{"resource":{"type":"teacher","id":"t_5b"},"maximum":6},{"resource":{"type":"class","id":"class_5v"},"maximum":6},{"resource":{"type":"teacher","id":"t_5v"},"maximum":6},{"resource":{"type":"class","id":"class_6a"},"maximum":6},{"resource":{"type":"teacher","id":"t_6a"},"maximum":6},{"resource":{"type":"class","id":"class_6b"},"maximum":6},{"resource":{"type":"teacher","id":"t_6b"},"maximum":6},{"resource":{"type":"class","id":"class_6v"},"maximum":6},{"resource":{"type":"teacher","id":"t_6v"},"maximum":6},{"resource":{"type":"class","id":"class_7a"},"maximum":7},{"resource":{"type":"teacher","id":"t_7a"},"maximum":7},{"resource":{"type":"class","id":"class_7b"},"maximum":7},{"resource":{"type":"teacher","id":"t_7b"},"maximum":7},{"resource":{"type":"class","id":"class_7v"},"maximum":7},{"resource":{"type":"teacher","id":"t_7v"},"maximum":7},{"resource":{"type":"class","id":"class_8a"},"maximum":7},{"resource":{"type":"teacher","id":"t_8a"},"maximum":7},{"resource":{"type":"class","id":"class_8b"},"maximum":7},{"resource":{"type":"teacher","id":"t_8b"},"maximum":7},{"resource":{"type":"class","id":"class_9a"},"maximum":7},{"resource":{"type":"teacher","id":"t_9a"},"maximum":7},{"resource":{"type":"class","id":"class_9b"},"maximum":7},{"resource":{"type":"teacher","id":"t_9b"},"maximum":7},{"resource":{"type":"class","id":"class_9v"},"maximum":7},{"resource":{"type":"teacher","id":"t_9v"},"maximum":7},{"resource":{"type":"class","id":"class_10a"},"maximum":7},{"resource":{"type":"teacher","id":"t_10a"},"maximum":7},{"resource":{"type":"class","id":"class_10b"},"maximum":7},{"resource":{"type":"teacher","id":"t_10b"},"maximum":7},{"resource":{"type":"class","id":"class_11a"},"maximum":7},{"resource":{"type":"teacher","id":"t_11a"},"maximum":7},{"resource":{"type":"class","id":"class_11b"},"maximum":7},{"resource":{"type":"teacher","id":"t_11b"},"maximum":7}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_5a"},"target":11},{"participant":{"type":"class","id":"class_5b"},"target":11},{"participant":{"type":"class","id":"class_5v"},"target":11},{"participant":{"type":"class","id":"class_6a"},"target":11},{"participant":{"type":"class","id":"class_6b"},"target":11},{"participant":{"type":"class","id":"class_6v"},"target":11},{"participant":{"type":"class","id":"class_7a"},"target":13},{"participant":{"type":"class","id":"class_7b"},"target":13},{"participant":{"type":"class","id":"class_7v"},"target":13},{"participant":{"type":"class","id":"class_8a"},"target":13},{"participant":{"type":"class","id":"class_8b"},"target":13},{"participant":{"type":"class","id":"class_9a"},"target":13},{"participant":{"type":"class","id":"class_9b"},"target":13},{"participant":{"type":"class","id":"class_9v"},"target":13},{"participant":{"type":"class","id":"class_10a"},"target":13},{"participant":{"type":"class","id":"class_10b"},"target":13},{"participant":{"type":"class","id":"class_11a"},"target":13},{"participant":{"type":"class","id":"class_11b"},"target":13}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P1","weight":40},{"constraint_id":"SC-003","priority":"P1","weight":200},{"constraint_id":"SC-004","priority":"P2","weight":3},{"constraint_id":"SC-005","priority":"P2","weight":4}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">

</xml_diff>

<commit_message>
feat: assign shared subject teachers
</commit_message>
<xml_diff>
--- a/outputs/stage-7/school-data-import-template.xlsx
+++ b/outputs/stage-7/school-data-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rab0dae508ed54259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="Rb8d2c5a50ffe46ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R22e712caeddd41f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" r:id="R66fc320b838647f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,12 +43,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -100,24 +105,25 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -333,88 +339,147 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="4" t="str">
         <x:v>ScheduleGenerator school data import</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-    </x:row>
-    <x:row r="2"/>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+    </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="7" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="7" t="str">
         <x:v>Action</x:v>
       </x:c>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="7" t="n">
+      <x:c r="A4" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B4" s="8" t="str">
         <x:v>Open the Dataset worksheet.</x:v>
       </x:c>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="7" t="n">
+      <x:c r="A5" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="str">
+      <x:c r="B5" s="8" t="str">
         <x:v>Edit JSON only in value_json. Keep every section name unique.</x:v>
       </x:c>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="7" t="n">
+      <x:c r="A6" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="8" t="str">
         <x:v>Save as .xlsx and run the import command in preview mode.</x:v>
       </x:c>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="7" t="n">
+      <x:c r="A7" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
+      <x:c r="B7" s="8" t="str">
         <x:v>Correct every reported row or field error.</x:v>
       </x:c>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1"/>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="7" t="n">
+      <x:c r="A8" s="8" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
+      <x:c r="B8" s="8" t="str">
         <x:v>Apply the same file only after the preview is valid.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9"/>
+      <x:c r="C8" s="1"/>
+      <x:c r="D8" s="1"/>
+      <x:c r="E8" s="1"/>
+      <x:c r="F8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="1"/>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1"/>
+      <x:c r="D9" s="1"/>
+      <x:c r="E9" s="1"/>
+      <x:c r="F9" s="1"/>
+    </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="10" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>Important: import is atomic. Invalid data is never partially saved.</x:v>
       </x:c>
-      <x:c r="B10" s="10"/>
-      <x:c r="C10" s="10"/>
-      <x:c r="D10" s="10"/>
-      <x:c r="E10" s="10"/>
-      <x:c r="F10" s="10"/>
+      <x:c r="B10" s="11"/>
+      <x:c r="C10" s="11"/>
+      <x:c r="D10" s="11"/>
+      <x:c r="E10" s="11"/>
+      <x:c r="F10" s="11"/>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="10" t="str">
+      <x:c r="A11" s="11" t="str">
         <x:v>The template contains synthetic demonstration data and no personal information.</x:v>
       </x:c>
-      <x:c r="B11" s="10"/>
-      <x:c r="C11" s="10"/>
-      <x:c r="D11" s="10"/>
-      <x:c r="E11" s="10"/>
-      <x:c r="F11" s="10"/>
-    </x:row>
-    <x:row r="12"/>
-    <x:row r="13"/>
-    <x:row r="14"/>
+      <x:c r="B11" s="11"/>
+      <x:c r="C11" s="11"/>
+      <x:c r="D11" s="11"/>
+      <x:c r="E11" s="11"/>
+      <x:c r="F11" s="11"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="1"/>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+      <x:c r="E12" s="1"/>
+      <x:c r="F12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="1"/>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1"/>
+      <x:c r="D13" s="1"/>
+      <x:c r="E13" s="1"/>
+      <x:c r="F13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+      <x:c r="E14" s="1"/>
+      <x:c r="F14" s="1"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -434,138 +499,138 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="13" t="str">
         <x:v>section</x:v>
       </x:c>
-      <x:c r="B1" s="12" t="str">
+      <x:c r="B1" s="13" t="str">
         <x:v>value_json</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="45" customHeight="1">
-      <x:c r="A2" s="16" t="str">
+      <x:c r="A2" s="17" t="str">
         <x:v>schema_version</x:v>
       </x:c>
-      <x:c r="B2" s="15" t="str">
+      <x:c r="B2" s="16" t="str">
         <x:v>"0.1.0"</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
-      <x:c r="A3" s="16" t="str">
+      <x:c r="A3" s="17" t="str">
         <x:v>dataset_id</x:v>
       </x:c>
-      <x:c r="B3" s="15" t="str">
+      <x:c r="B3" s="16" t="str">
         <x:v>"small_school_demo"</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
-      <x:c r="A4" s="16" t="str">
+      <x:c r="A4" s="17" t="str">
         <x:v>school</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="str">
+      <x:c r="B4" s="16" t="str">
         <x:v>{"id":"demo_school","label":"Representative Demonstration School","timezone":"Europe/Minsk"}</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
-      <x:c r="A5" s="16" t="str">
+      <x:c r="A5" s="17" t="str">
         <x:v>academic_period</x:v>
       </x:c>
-      <x:c r="B5" s="15" t="str">
+      <x:c r="B5" s="16" t="str">
         <x:v>{"id":"term_1_2026","label":"Demonstration Term 1","start_date":"2026-09-01","end_date":"2026-12-24","days":[{"id":"mon","label":"Monday","ordinal":1},{"id":"tue","label":"Tuesday","ordinal":2},{"id":"wed","label":"Wednesday","ordinal":3},{"id":"thu","label":"Thursday","ordinal":4},{"id":"fri","label":"Friday","ordinal":5}],"periods":[{"id":"p1","label":"Period 1","ordinal":1,"start_time":"08:00","end_time":"08:45"},{"id":"p2","label":"Period 2","ordinal":2,"start_time":"08:55","end_time":"09:40"},{"id":"p3","label":"Period 3","ordinal":3,"start_time":"10:00","end_time":"10:45"},{"id":"p4","label":"Period 4","ordinal":4,"start_time":"11:05","end_time":"11:50"},{"id":"p5","label":"Period 5","ordinal":5,"start_time":"12:00","end_time":"12:45"},{"id":"p6","label":"Period 6","ordinal":6,"start_time":"12:55","end_time":"13:40"},{"id":"p7","label":"Period 7","ordinal":7,"start_time":"13:50","end_time":"14:35"}],"shifts":[{"id":"morning","label":"Morning shift","period_ids":["p1","p2","p3","p4","p5","p6","p7"]}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
-      <x:c r="A6" s="16" t="str">
+      <x:c r="A6" s="17" t="str">
         <x:v>subjects</x:v>
       </x:c>
-      <x:c r="B6" s="15" t="str">
+      <x:c r="B6" s="16" t="str">
         <x:v>[{"id":"mathematics","label":"Mathematics","default_workload":3},{"id":"russian_language","label":"Russian Language","default_workload":3},{"id":"russian_literature","label":"Russian Literature","default_workload":2},{"id":"belarusian_language","label":"Belarusian Language","default_workload":3},{"id":"belarusian_literature","label":"Belarusian Literature","default_workload":2},{"id":"english","label":"English","default_workload":2},{"id":"physical_education","label":"Physical Education","default_workload":1},{"id":"technology","label":"Technology","default_workload":1},{"id":"informatics","label":"Informatics","default_workload":2},{"id":"art","label":"Art","default_workload":1},{"id":"human_and_world","label":"Human and the World","default_workload":1},{"id":"life_safety","label":"Life Safety","default_workload":1},{"id":"biology","label":"Biology","default_workload":3},{"id":"geography","label":"Geography","default_workload":2},{"id":"history_belarus","label":"History of Belarus","default_workload":2},{"id":"world_history","label":"World History","default_workload":2},{"id":"physics","label":"Physics","default_workload":3},{"id":"chemistry","label":"Chemistry","default_workload":3},{"id":"social_studies","label":"Social Studies","default_workload":2},{"id":"technical_drawing","label":"Technical Drawing","default_workload":2},{"id":"astronomy","label":"Astronomy","default_workload":3},{"id":"defense_medical","label":"Defense and Medical Training","default_workload":1}]</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
-      <x:c r="A7" s="16" t="str">
+      <x:c r="A7" s="17" t="str">
         <x:v>teachers</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="str">
-        <x:v>[{"id":"t_math","label":"Teacher T-5A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_5b","label":"Teacher T-5B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_5v","label":"Teacher T-5V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6a","label":"Teacher T-6A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6b","label":"Teacher T-6B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_6v","label":"Teacher T-6V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7a","label":"Teacher T-7A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7b","label":"Teacher T-7B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_7v","label":"Teacher T-7V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_8a","label":"Teacher T-8A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_8b","label":"Teacher T-8B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9a","label":"Teacher T-9A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9b","label":"Teacher T-9B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_9v","label":"Teacher T-9V","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_10a","label":"Teacher T-10A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_10b","label":"Teacher T-10B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_11a","label":"Teacher T-11A","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_11b","label":"Teacher T-11B","qualified_subject_ids":["mathematics","russian_language","russian_literature","belarusian_language","belarusian_literature","english","physical_education","technology","informatics","art","human_and_world","life_safety","biology","geography","history_belarus","world_history","physics","chemistry","social_studies","technical_drawing","astronomy","defense_medical"]},{"id":"t_science","label":"Teacher T-Science","qualified_subject_ids":["physics","chemistry"]},{"id":"t_english_a","label":"Teacher T-English-A","qualified_subject_ids":["english"]},{"id":"t_english_b","label":"Teacher T-English-B","qualified_subject_ids":["english"]},{"id":"t_history","label":"Teacher T-History","qualified_subject_ids":["art"]}]</x:v>
+      <x:c r="B7" s="16" t="str">
+        <x:v>[{"id":"t_math","label":"Smirnov","qualified_subject_ids":["mathematics"]},{"id":"t_math_2","label":"Kuznetsova","qualified_subject_ids":["mathematics"]},{"id":"t_math_3","label":"Sokolov","qualified_subject_ids":["mathematics"]},{"id":"t_math_4","label":"Volkova","qualified_subject_ids":["mathematics"]},{"id":"t_math_5","label":"Popov","qualified_subject_ids":["mathematics"]},{"id":"t_math_6","label":"Medvedeva","qualified_subject_ids":["mathematics"]},{"id":"t_math_7","label":"Denisov","qualified_subject_ids":["mathematics"]},{"id":"t_russian_1","label":"Ivanov","qualified_subject_ids":["russian_language","russian_literature"]},{"id":"t_russian_2","label":"Morozova","qualified_subject_ids":["russian_language","russian_literature"]},{"id":"t_russian_3","label":"Lebedev","qualified_subject_ids":["russian_language","russian_literature"]},{"id":"t_belarusian_1","label":"Kovalenko","qualified_subject_ids":["belarusian_language","belarusian_literature"]},{"id":"t_belarusian_2","label":"Shevchenko","qualified_subject_ids":["belarusian_language","belarusian_literature"]},{"id":"t_belarusian_3","label":"Bondarenko","qualified_subject_ids":["belarusian_language","belarusian_literature"]},{"id":"t_english_1","label":"Taylor","qualified_subject_ids":["english"]},{"id":"t_english_2","label":"Brown","qualified_subject_ids":["english"]},{"id":"t_english_3","label":"Wilson","qualified_subject_ids":["english"]},{"id":"t_english_4","label":"Cooper","qualified_subject_ids":["english"]},{"id":"t_english_5","label":"Harris","qualified_subject_ids":["english"]},{"id":"t_english_6","label":"Martin","qualified_subject_ids":["english"]},{"id":"t_pe_1","label":"Orlov","qualified_subject_ids":["physical_education"]},{"id":"t_pe_2","label":"Pavlova","qualified_subject_ids":["physical_education"]},{"id":"t_pe_3","label":"Zaitsev","qualified_subject_ids":["physical_education"]},{"id":"t_pe_4","label":"Karpov","qualified_subject_ids":["physical_education"]},{"id":"t_pe_5","label":"Kulikov","qualified_subject_ids":["physical_education"]},{"id":"t_physics","label":"Fedorov","qualified_subject_ids":["physics","astronomy"]},{"id":"t_physics_2","label":"Vinogradov","qualified_subject_ids":["physics","astronomy"]},{"id":"t_chemistry","label":"Mikhailova","qualified_subject_ids":["chemistry"]},{"id":"t_chemistry_2","label":"Belyaeva","qualified_subject_ids":["chemistry"]},{"id":"t_biology","label":"Egorova","qualified_subject_ids":["biology"]},{"id":"t_biology_2","label":"Nikolaeva","qualified_subject_ids":["biology"]},{"id":"t_biology_3","label":"Alexeev","qualified_subject_ids":["biology"]},{"id":"t_belarus_history","label":"Novik","qualified_subject_ids":["history_belarus"]},{"id":"t_belarus_history_2","label":"Kravchenko","qualified_subject_ids":["history_belarus"]},{"id":"t_belarus_history_3","label":"Savchenko","qualified_subject_ids":["history_belarus"]},{"id":"t_world_history","label":"Romanov","qualified_subject_ids":["world_history"]},{"id":"t_world_history_2","label":"Semenov","qualified_subject_ids":["world_history"]},{"id":"t_world_history_3","label":"Gromov","qualified_subject_ids":["world_history"]},{"id":"t_geography","label":"Kozlova","qualified_subject_ids":["geography","social_studies"]},{"id":"t_geography_2","label":"Sorokina","qualified_subject_ids":["geography","social_studies"]},{"id":"t_geography_3","label":"Vasiliev","qualified_subject_ids":["geography","social_studies"]},{"id":"t_technology","label":"Andreev","qualified_subject_ids":["technology","technical_drawing"]},{"id":"t_technology_2","label":"Tarasov","qualified_subject_ids":["technology","technical_drawing"]},{"id":"t_technology_3","label":"Bogdanov","qualified_subject_ids":["technology","technical_drawing"]},{"id":"t_art","label":"Petrov","qualified_subject_ids":["art","human_and_world","life_safety"]},{"id":"t_art_2","label":"Golubeva","qualified_subject_ids":["art","human_and_world","life_safety"]},{"id":"t_art_3","label":"Komarov","qualified_subject_ids":["art","human_and_world","life_safety"]},{"id":"t_art_4","label":"Fomina","qualified_subject_ids":["art","human_and_world","life_safety"]},{"id":"t_informatics","label":"Markov","qualified_subject_ids":["informatics"]},{"id":"t_informatics_2","label":"Zhukov","qualified_subject_ids":["informatics"]},{"id":"t_informatics_3","label":"Kiselev","qualified_subject_ids":["informatics"]},{"id":"t_defense","label":"Belov","qualified_subject_ids":["defense_medical"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
-      <x:c r="A8" s="16" t="str">
+      <x:c r="A8" s="17" t="str">
         <x:v>classrooms</x:v>
       </x:c>
-      <x:c r="B8" s="15" t="str">
-        <x:v>[{"id":"room_5a","label":"Room 5A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5b","label":"Room 5B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5v","label":"Room 5V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6a","label":"Room 6A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6b","label":"Room 6B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6v","label":"Room 6V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7a","label":"Room 7A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7b","label":"Room 7B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7v","label":"Room 7V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8a","label":"Room 8A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8b","label":"Room 8B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9a","label":"Room 9A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9b","label":"Room 9B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9v","label":"Room 9V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10a","label":"Room 10A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10b","label":"Room 10B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11a","label":"Room 11A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11b","label":"Room 11B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"science_lab","label":"Science Laboratory","capacity":30,"capabilities":["general","physics_lab","chemistry_lab"]},{"id":"hall","label":"Assembly Hall","capacity":60,"capabilities":["assembly"]},{"id":"language_room_a","label":"Language Room A","capacity":30,"capabilities":["general"]},{"id":"language_room_b","label":"Language Room B","capacity":30,"capabilities":["general"]}]</x:v>
+      <x:c r="B8" s="16" t="str">
+        <x:v>[{"id":"room_5a","label":"Room 5A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5b","label":"Room 5B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_5v","label":"Room 5V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6a","label":"Room 6A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6b","label":"Room 6B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_6v","label":"Room 6V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7a","label":"Room 7A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7b","label":"Room 7B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_7v","label":"Room 7V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8a","label":"Room 8A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_8b","label":"Room 8B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9a","label":"Room 9A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9b","label":"Room 9B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_9v","label":"Room 9V","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10a","label":"Room 10A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_10b","label":"Room 10B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11a","label":"Room 11A","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]},{"id":"room_11b","label":"Room 11B","capacity":30,"capabilities":["general","sports","physics_lab","chemistry_lab","computer_lab","workshop","art"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="45" customHeight="1">
-      <x:c r="A9" s="16" t="str">
+      <x:c r="A9" s="17" t="str">
         <x:v>classes</x:v>
       </x:c>
-      <x:c r="B9" s="15" t="str">
+      <x:c r="B9" s="16" t="str">
         <x:v>[{"id":"class_5a","label":"Class 5A","grade":5,"student_count":26,"shift_id":"morning"},{"id":"class_5b","label":"Class 5B","grade":5,"student_count":27,"shift_id":"morning"},{"id":"class_5v","label":"Class 5V","grade":5,"student_count":27,"shift_id":"morning"},{"id":"class_6a","label":"Class 6A","grade":6,"student_count":27,"shift_id":"morning"},{"id":"class_6b","label":"Class 6B","grade":6,"student_count":28,"shift_id":"morning"},{"id":"class_6v","label":"Class 6V","grade":6,"student_count":28,"shift_id":"morning"},{"id":"class_7a","label":"Class 7A","grade":7,"student_count":28,"shift_id":"morning"},{"id":"class_7b","label":"Class 7B","grade":7,"student_count":24,"shift_id":"morning"},{"id":"class_7v","label":"Class 7V","grade":7,"student_count":24,"shift_id":"morning"},{"id":"class_8a","label":"Class 8A","grade":8,"student_count":24,"shift_id":"morning"},{"id":"class_8b","label":"Class 8B","grade":8,"student_count":25,"shift_id":"morning"},{"id":"class_9a","label":"Class 9A","grade":9,"student_count":25,"shift_id":"morning"},{"id":"class_9b","label":"Class 9B","grade":9,"student_count":26,"shift_id":"morning"},{"id":"class_9v","label":"Class 9V","grade":9,"student_count":26,"shift_id":"morning"},{"id":"class_10a","label":"Class 10A","grade":10,"student_count":26,"shift_id":"morning"},{"id":"class_10b","label":"Class 10B","grade":10,"student_count":27,"shift_id":"morning"},{"id":"class_11a","label":"Class 11A","grade":11,"student_count":27,"shift_id":"morning"},{"id":"class_11b","label":"Class 11B","grade":11,"student_count":28,"shift_id":"morning"}]</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="45" customHeight="1">
-      <x:c r="A10" s="16" t="str">
+      <x:c r="A10" s="17" t="str">
         <x:v>group_partitions</x:v>
       </x:c>
-      <x:c r="B10" s="15" t="str">
+      <x:c r="B10" s="16" t="str">
         <x:v>[{"id":"partition_7a_english","label":"Class 7A English groups","class_id":"class_7a","complete":true}]</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="45" customHeight="1">
-      <x:c r="A11" s="16" t="str">
+      <x:c r="A11" s="17" t="str">
         <x:v>groups</x:v>
       </x:c>
-      <x:c r="B11" s="15" t="str">
+      <x:c r="B11" s="16" t="str">
         <x:v>[{"id":"group_7a_en_1","label":"Class 7A English Group 1","class_id":"class_7a","partition_id":"partition_7a_english","student_count":14},{"id":"group_7a_en_2","label":"Class 7A English Group 2","class_id":"class_7a","partition_id":"partition_7a_english","student_count":14}]</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
-      <x:c r="A12" s="16" t="str">
+      <x:c r="A12" s="17" t="str">
         <x:v>cohorts</x:v>
       </x:c>
-      <x:c r="B12" s="15" t="str">
+      <x:c r="B12" s="16" t="str">
         <x:v>[{"id":"cohort_7a_8a_advisory","label":"Classes 7A and 8A Advisory","members":[{"type":"class","id":"class_7a"},{"type":"class","id":"class_8a"}]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="45" customHeight="1">
-      <x:c r="A13" s="16" t="str">
+      <x:c r="A13" s="17" t="str">
         <x:v>curriculum_requirements</x:v>
       </x:c>
-      <x:c r="B13" s="15" t="str">
-        <x:v>[{"id":"req_5a_mathematics","participant":{"type":"class","id":"class_5a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_language","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_english","participant":{"type":"class","id":"class_5a"},"subject_id":"english","eligible_teacher_ids":["t_math"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_physical_education","participant":{"type":"class","id":"class_5a"},"subject_id":"physical_education","eligible_teacher_ids":["t_math"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_technology","participant":{"type":"class","id":"class_5a"},"subject_id":"technology","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_art","participant":{"type":"class","id":"class_5a"},"subject_id":"art","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_human_and_world","participant":{"type":"class","id":"class_5a"},"subject_id":"human_and_world","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_life_safety","participant":{"type":"class","id":"class_5a"},"subject_id":"life_safety","eligible_teacher_ids":["t_math"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_world_history","participant":{"type":"class","id":"class_5a"},"subject_id":"world_history","eligible_teacher_ids":["t_math"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5b_mathematics","participant":{"type":"class","id":"class_5b"},"subject_id":"mathematics","eligible_teacher_ids":["t_5b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_language","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_english","participant":{"type":"class","id":"class_5b"},"subject_id":"english","eligible_teacher_ids":["t_5b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_physical_education","participant":{"type":"class","id":"class_5b"},"subject_id":"physical_education","eligible_teacher_ids":["t_5b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_technology","participant":{"type":"class","id":"class_5b"},"subject_id":"technology","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_art","participant":{"type":"class","id":"class_5b"},"subject_id":"art","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_human_and_world","participant":{"type":"class","id":"class_5b"},"subject_id":"human_and_world","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_life_safety","participant":{"type":"class","id":"class_5b"},"subject_id":"life_safety","eligible_teacher_ids":["t_5b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_world_history","participant":{"type":"class","id":"class_5b"},"subject_id":"world_history","eligible_teacher_ids":["t_5b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5v_mathematics","participant":{"type":"class","id":"class_5v"},"subject_id":"mathematics","eligible_teacher_ids":["t_5v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_language","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_english","participant":{"type":"class","id":"class_5v"},"subject_id":"english","eligible_teacher_ids":["t_5v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_physical_education","participant":{"type":"class","id":"class_5v"},"subject_id":"physical_education","eligible_teacher_ids":["t_5v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_technology","participant":{"type":"class","id":"class_5v"},"subject_id":"technology","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_art","participant":{"type":"class","id":"class_5v"},"subject_id":"art","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_human_and_world","participant":{"type":"class","id":"class_5v"},"subject_id":"human_and_world","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_life_safety","participant":{"type":"class","id":"class_5v"},"subject_id":"life_safety","eligible_teacher_ids":["t_5v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_world_history","participant":{"type":"class","id":"class_5v"},"subject_id":"world_history","eligible_teacher_ids":["t_5v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_6a_mathematics","participant":{"type":"class","id":"class_6a"},"subject_id":"mathematics","eligible_teacher_ids":["t_6a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_language","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_english","participant":{"type":"class","id":"class_6a"},"subject_id":"english","eligible_teacher_ids":["t_6a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_physical_education","participant":{"type":"class","id":"class_6a"},"subject_id":"physical_education","eligible_teacher_ids":["t_6a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_technology","participant":{"type":"class","id":"class_6a"},"subject_id":"technology","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_informatics","participant":{"type":"class","id":"class_6a"},"subject_id":"informatics","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_art","participant":{"type":"class","id":"class_6a"},"subject_id":"art","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_biology","participant":{"type":"class","id":"class_6a"},"subject_id":"biology","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_geography","participant":{"type":"class","id":"class_6a"},"subject_id":"geography","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_history_belarus","participant":{"type":"class","id":"class_6a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_world_history","participant":{"type":"class","id":"class_6a"},"subject_id":"world_history","eligible_teacher_ids":["t_6a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6b_mathematics","participant":{"type":"class","id":"class_6b"},"subject_id":"mathematics","eligible_teacher_ids":["t_6b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_language","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_english","participant":{"type":"class","id":"class_6b"},"subject_id":"english","eligible_teacher_ids":["t_6b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_physical_education","participant":{"type":"class","id":"class_6b"},"subject_id":"physical_education","eligible_teacher_ids":["t_6b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_technology","participant":{"type":"class","id":"class_6b"},"subject_id":"technology","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_informatics","participant":{"type":"class","id":"class_6b"},"subject_id":"informatics","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_art","participant":{"type":"class","id":"class_6b"},"subject_id":"art","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_biology","participant":{"type":"class","id":"class_6b"},"subject_id":"biology","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_geography","participant":{"type":"class","id":"class_6b"},"subject_id":"geography","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_history_belarus","participant":{"type":"class","id":"class_6b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_world_history","participant":{"type":"class","id":"class_6b"},"subject_id":"world_history","eligible_teacher_ids":["t_6b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6v_mathematics","participant":{"type":"class","id":"class_6v"},"subject_id":"mathematics","eligible_teacher_ids":["t_6v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_language","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_6v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_6v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_english","participant":{"type":"class","id":"class_6v"},"subject_id":"english","eligible_teacher_ids":["t_6v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_physical_education","participant":{"type":"class","id":"class_6v"},"subject_id":"physical_education","eligible_teacher_ids":["t_6v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_technology","participant":{"type":"class","id":"class_6v"},"subject_id":"technology","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_informatics","participant":{"type":"class","id":"class_6v"},"subject_id":"informatics","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_art","participant":{"type":"class","id":"class_6v"},"subject_id":"art","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_biology","participant":{"type":"class","id":"class_6v"},"subject_id":"biology","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_geography","participant":{"type":"class","id":"class_6v"},"subject_id":"geography","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_history_belarus","participant":{"type":"class","id":"class_6v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_world_history","participant":{"type":"class","id":"class_6v"},"subject_id":"world_history","eligible_teacher_ids":["t_6v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_7a_math","participant":{"type":"class","id":"class_7a"},"subject_id":"mathematics","eligible_teacher_ids":["t_7a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_language","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_en_1","participant":{"type":"class","id":"class_7a"},"subject_id":"english","eligible_teacher_ids":["t_7a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physical_education","participant":{"type":"class","id":"class_7a"},"subject_id":"physical_education","eligible_teacher_ids":["t_7a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_technology","participant":{"type":"class","id":"class_7a"},"subject_id":"technology","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_informatics","participant":{"type":"class","id":"class_7a"},"subject_id":"informatics","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_joint_advisory","participant":{"type":"class","id":"class_7a"},"subject_id":"art","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_biology","participant":{"type":"class","id":"class_7a"},"subject_id":"biology","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_geography","participant":{"type":"class","id":"class_7a"},"subject_id":"geography","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_history_belarus","participant":{"type":"class","id":"class_7a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_world_history","participant":{"type":"class","id":"class_7a"},"subject_id":"world_history","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physics","participant":{"type":"class","id":"class_7a"},"subject_id":"physics","eligible_teacher_ids":["t_7a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_chemistry","participant":{"type":"class","id":"class_7a"},"subject_id":"chemistry","eligible_teacher_ids":["t_7a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7b_mathematics","participant":{"type":"class","id":"class_7b"},"subject_id":"mathematics","eligible_teacher_ids":["t_7b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_language","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_english","participant":{"type":"class","id":"class_7b"},"subject_id":"english","eligible_teacher_ids":["t_7b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physical_education","participant":{"type":"class","id":"class_7b"},"subject_id":"physical_education","eligible_teacher_ids":["t_7b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_technology","participant":{"type":"class","id":"class_7b"},"subject_id":"technology","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_informatics","participant":{"type":"class","id":"class_7b"},"subject_id":"informatics","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_art","participant":{"type":"class","id":"class_7b"},"subject_id":"art","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_biology","participant":{"type":"class","id":"class_7b"},"subject_id":"biology","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_geography","participant":{"type":"class","id":"class_7b"},"subject_id":"geography","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_history_belarus","participant":{"type":"class","id":"class_7b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_world_history","participant":{"type":"class","id":"class_7b"},"subject_id":"world_history","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physics","participant":{"type":"class","id":"class_7b"},"subject_id":"physics","eligible_teacher_ids":["t_7b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_chemistry","participant":{"type":"class","id":"class_7b"},"subject_id":"chemistry","eligible_teacher_ids":["t_7b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7v_mathematics","participant":{"type":"class","id":"class_7v"},"subject_id":"mathematics","eligible_teacher_ids":["t_7v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_language","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_english","participant":{"type":"class","id":"class_7v"},"subject_id":"english","eligible_teacher_ids":["t_7v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physical_education","participant":{"type":"class","id":"class_7v"},"subject_id":"physical_education","eligible_teacher_ids":["t_7v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_technology","participant":{"type":"class","id":"class_7v"},"subject_id":"technology","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_informatics","participant":{"type":"class","id":"class_7v"},"subject_id":"informatics","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_art","participant":{"type":"class","id":"class_7v"},"subject_id":"art","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_biology","participant":{"type":"class","id":"class_7v"},"subject_id":"biology","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_geography","participant":{"type":"class","id":"class_7v"},"subject_id":"geography","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_history_belarus","participant":{"type":"class","id":"class_7v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_world_history","participant":{"type":"class","id":"class_7v"},"subject_id":"world_history","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physics","participant":{"type":"class","id":"class_7v"},"subject_id":"physics","eligible_teacher_ids":["t_7v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_chemistry","participant":{"type":"class","id":"class_7v"},"subject_id":"chemistry","eligible_teacher_ids":["t_7v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_8a_mathematics","participant":{"type":"class","id":"class_8a"},"subject_id":"mathematics","eligible_teacher_ids":["t_8a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_language","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_english","participant":{"type":"class","id":"class_8a"},"subject_id":"english","eligible_teacher_ids":["t_8a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physical_education","participant":{"type":"class","id":"class_8a"},"subject_id":"physical_education","eligible_teacher_ids":["t_8a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_technology","participant":{"type":"class","id":"class_8a"},"subject_id":"technology","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_informatics","participant":{"type":"class","id":"class_8a"},"subject_id":"informatics","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_art","participant":{"type":"class","id":"class_8a"},"subject_id":"art","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_biology","participant":{"type":"class","id":"class_8a"},"subject_id":"biology","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_geography","participant":{"type":"class","id":"class_8a"},"subject_id":"geography","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_history_belarus","participant":{"type":"class","id":"class_8a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_world_history","participant":{"type":"class","id":"class_8a"},"subject_id":"world_history","eligible_teacher_ids":["t_8a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physics","participant":{"type":"class","id":"class_8a"},"subject_id":"physics","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_chemistry","participant":{"type":"class","id":"class_8a"},"subject_id":"chemistry","eligible_teacher_ids":["t_8a"],"weekly_lessons":2,"block_length":2,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8b_mathematics","participant":{"type":"class","id":"class_8b"},"subject_id":"mathematics","eligible_teacher_ids":["t_8b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_language","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_english","participant":{"type":"class","id":"class_8b"},"subject_id":"english","eligible_teacher_ids":["t_8b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physical_education","participant":{"type":"class","id":"class_8b"},"subject_id":"physical_education","eligible_teacher_ids":["t_8b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_technology","participant":{"type":"class","id":"class_8b"},"subject_id":"technology","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_informatics","participant":{"type":"class","id":"class_8b"},"subject_id":"informatics","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_art","participant":{"type":"class","id":"class_8b"},"subject_id":"art","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_biology","participant":{"type":"class","id":"class_8b"},"subject_id":"biology","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_geography","participant":{"type":"class","id":"class_8b"},"subject_id":"geography","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_history_belarus","participant":{"type":"class","id":"class_8b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_world_history","participant":{"type":"class","id":"class_8b"},"subject_id":"world_history","eligible_teacher_ids":["t_8b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physics","participant":{"type":"class","id":"class_8b"},"subject_id":"physics","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_chemistry","participant":{"type":"class","id":"class_8b"},"subject_id":"chemistry","eligible_teacher_ids":["t_8b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_9a_mathematics","participant":{"type":"class","id":"class_9a"},"subject_id":"mathematics","eligible_teacher_ids":["t_9a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_language","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_english","participant":{"type":"class","id":"class_9a"},"subject_id":"english","eligible_teacher_ids":["t_9a"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physical_education","participant":{"type":"class","id":"class_9a"},"subject_id":"physical_education","eligible_teacher_ids":["t_9a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_technology","participant":{"type":"class","id":"class_9a"},"subject_id":"technology","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_informatics","participant":{"type":"class","id":"class_9a"},"subject_id":"informatics","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_biology","participant":{"type":"class","id":"class_9a"},"subject_id":"biology","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_geography","participant":{"type":"class","id":"class_9a"},"subject_id":"geography","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_history_belarus","participant":{"type":"class","id":"class_9a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_world_history","participant":{"type":"class","id":"class_9a"},"subject_id":"world_history","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physics","participant":{"type":"class","id":"class_9a"},"subject_id":"physics","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_chemistry","participant":{"type":"class","id":"class_9a"},"subject_id":"chemistry","eligible_teacher_ids":["t_9a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_social_studies","participant":{"type":"class","id":"class_9a"},"subject_id":"social_studies","eligible_teacher_ids":["t_9a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9b_mathematics","participant":{"type":"class","id":"class_9b"},"subject_id":"mathematics","eligible_teacher_ids":["t_9b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_language","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_english","participant":{"type":"class","id":"class_9b"},"subject_id":"english","eligible_teacher_ids":["t_9b"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physical_education","participant":{"type":"class","id":"class_9b"},"subject_id":"physical_education","eligible_teacher_ids":["t_9b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_technology","participant":{"type":"class","id":"class_9b"},"subject_id":"technology","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_informatics","participant":{"type":"class","id":"class_9b"},"subject_id":"informatics","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_biology","participant":{"type":"class","id":"class_9b"},"subject_id":"biology","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_geography","participant":{"type":"class","id":"class_9b"},"subject_id":"geography","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_history_belarus","participant":{"type":"class","id":"class_9b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_world_history","participant":{"type":"class","id":"class_9b"},"subject_id":"world_history","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physics","participant":{"type":"class","id":"class_9b"},"subject_id":"physics","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_chemistry","participant":{"type":"class","id":"class_9b"},"subject_id":"chemistry","eligible_teacher_ids":["t_9b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_social_studies","participant":{"type":"class","id":"class_9b"},"subject_id":"social_studies","eligible_teacher_ids":["t_9b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9v_mathematics","participant":{"type":"class","id":"class_9v"},"subject_id":"mathematics","eligible_teacher_ids":["t_9v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_language","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_english","participant":{"type":"class","id":"class_9v"},"subject_id":"english","eligible_teacher_ids":["t_9v"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physical_education","participant":{"type":"class","id":"class_9v"},"subject_id":"physical_education","eligible_teacher_ids":["t_9v"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_technology","participant":{"type":"class","id":"class_9v"},"subject_id":"technology","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_informatics","participant":{"type":"class","id":"class_9v"},"subject_id":"informatics","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_biology","participant":{"type":"class","id":"class_9v"},"subject_id":"biology","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_geography","participant":{"type":"class","id":"class_9v"},"subject_id":"geography","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_history_belarus","participant":{"type":"class","id":"class_9v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_world_history","participant":{"type":"class","id":"class_9v"},"subject_id":"world_history","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physics","participant":{"type":"class","id":"class_9v"},"subject_id":"physics","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_chemistry","participant":{"type":"class","id":"class_9v"},"subject_id":"chemistry","eligible_teacher_ids":["t_9v"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_social_studies","participant":{"type":"class","id":"class_9v"},"subject_id":"social_studies","eligible_teacher_ids":["t_9v"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_10a_mathematics","participant":{"type":"class","id":"class_10a"},"subject_id":"mathematics","eligible_teacher_ids":["t_10a"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physics","participant":{"type":"class","id":"class_10a"},"subject_id":"physics","eligible_teacher_ids":["t_10a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_chemistry","participant":{"type":"class","id":"class_10a"},"subject_id":"chemistry","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_biology","participant":{"type":"class","id":"class_10a"},"subject_id":"biology","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_language","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_english","participant":{"type":"class","id":"class_10a"},"subject_id":"english","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physical_education","participant":{"type":"class","id":"class_10a"},"subject_id":"physical_education","eligible_teacher_ids":["t_10a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_informatics","participant":{"type":"class","id":"class_10a"},"subject_id":"informatics","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_geography","participant":{"type":"class","id":"class_10a"},"subject_id":"geography","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_history_belarus","participant":{"type":"class","id":"class_10a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_10a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_social_studies","participant":{"type":"class","id":"class_10a"},"subject_id":"social_studies","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_technical_drawing","participant":{"type":"class","id":"class_10a"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_defense_medical","participant":{"type":"class","id":"class_10a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_10a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10b_mathematics","participant":{"type":"class","id":"class_10b"},"subject_id":"mathematics","eligible_teacher_ids":["t_10b"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physics","participant":{"type":"class","id":"class_10b"},"subject_id":"physics","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_chemistry","participant":{"type":"class","id":"class_10b"},"subject_id":"chemistry","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_biology","participant":{"type":"class","id":"class_10b"},"subject_id":"biology","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_language","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_english","participant":{"type":"class","id":"class_10b"},"subject_id":"english","eligible_teacher_ids":["t_10b"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physical_education","participant":{"type":"class","id":"class_10b"},"subject_id":"physical_education","eligible_teacher_ids":["t_10b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_informatics","participant":{"type":"class","id":"class_10b"},"subject_id":"informatics","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_geography","participant":{"type":"class","id":"class_10b"},"subject_id":"geography","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_history_belarus","participant":{"type":"class","id":"class_10b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_10b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_social_studies","participant":{"type":"class","id":"class_10b"},"subject_id":"social_studies","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_technical_drawing","participant":{"type":"class","id":"class_10b"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_defense_medical","participant":{"type":"class","id":"class_10b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_10b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_11a_mathematics","participant":{"type":"class","id":"class_11a"},"subject_id":"mathematics","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physics","participant":{"type":"class","id":"class_11a"},"subject_id":"physics","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_chemistry","participant":{"type":"class","id":"class_11a"},"subject_id":"chemistry","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_biology","participant":{"type":"class","id":"class_11a"},"subject_id":"biology","eligible_teacher_ids":["t_11a"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_language","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_english","participant":{"type":"class","id":"class_11a"},"subject_id":"english","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physical_education","participant":{"type":"class","id":"class_11a"},"subject_id":"physical_education","eligible_teacher_ids":["t_11a"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_informatics","participant":{"type":"class","id":"class_11a"},"subject_id":"informatics","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_geography","participant":{"type":"class","id":"class_11a"},"subject_id":"geography","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_history_belarus","participant":{"type":"class","id":"class_11a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_11a"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_social_studies","participant":{"type":"class","id":"class_11a"},"subject_id":"social_studies","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_astronomy","participant":{"type":"class","id":"class_11a"},"subject_id":"astronomy","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_defense_medical","participant":{"type":"class","id":"class_11a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_11a"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11b_mathematics","participant":{"type":"class","id":"class_11b"},"subject_id":"mathematics","eligible_teacher_ids":["t_11b"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physics","participant":{"type":"class","id":"class_11b"},"subject_id":"physics","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_chemistry","participant":{"type":"class","id":"class_11b"},"subject_id":"chemistry","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_biology","participant":{"type":"class","id":"class_11b"},"subject_id":"biology","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_language","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_english","participant":{"type":"class","id":"class_11b"},"subject_id":"english","eligible_teacher_ids":["t_11b"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physical_education","participant":{"type":"class","id":"class_11b"},"subject_id":"physical_education","eligible_teacher_ids":["t_11b"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_informatics","participant":{"type":"class","id":"class_11b"},"subject_id":"informatics","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_geography","participant":{"type":"class","id":"class_11b"},"subject_id":"geography","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_history_belarus","participant":{"type":"class","id":"class_11b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_11b"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_social_studies","participant":{"type":"class","id":"class_11b"},"subject_id":"social_studies","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_astronomy","participant":{"type":"class","id":"class_11b"},"subject_id":"astronomy","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_defense_medical","participant":{"type":"class","id":"class_11b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_11b"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]}]</x:v>
+      <x:c r="B13" s="16" t="str">
+        <x:v>[{"id":"req_5a_mathematics","participant":{"type":"class","id":"class_5a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_russian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_language","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_belarusian_literature","participant":{"type":"class","id":"class_5a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_english","participant":{"type":"class","id":"class_5a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_physical_education","participant":{"type":"class","id":"class_5a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_technology","participant":{"type":"class","id":"class_5a"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_art","participant":{"type":"class","id":"class_5a"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_human_and_world","participant":{"type":"class","id":"class_5a"},"subject_id":"human_and_world","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_life_safety","participant":{"type":"class","id":"class_5a"},"subject_id":"life_safety","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5a_world_history","participant":{"type":"class","id":"class_5a"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5a"]},{"id":"req_5b_mathematics","participant":{"type":"class","id":"class_5b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_russian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_language","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_belarusian_literature","participant":{"type":"class","id":"class_5b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_english","participant":{"type":"class","id":"class_5b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_physical_education","participant":{"type":"class","id":"class_5b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_technology","participant":{"type":"class","id":"class_5b"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_art","participant":{"type":"class","id":"class_5b"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_human_and_world","participant":{"type":"class","id":"class_5b"},"subject_id":"human_and_world","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_life_safety","participant":{"type":"class","id":"class_5b"},"subject_id":"life_safety","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5b_world_history","participant":{"type":"class","id":"class_5b"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5b"]},{"id":"req_5v_mathematics","participant":{"type":"class","id":"class_5v"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_russian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_language","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_belarusian_literature","participant":{"type":"class","id":"class_5v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_english","participant":{"type":"class","id":"class_5v"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_physical_education","participant":{"type":"class","id":"class_5v"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_technology","participant":{"type":"class","id":"class_5v"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_art","participant":{"type":"class","id":"class_5v"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_human_and_world","participant":{"type":"class","id":"class_5v"},"subject_id":"human_and_world","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_life_safety","participant":{"type":"class","id":"class_5v"},"subject_id":"life_safety","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_5v_world_history","participant":{"type":"class","id":"class_5v"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_5v"]},{"id":"req_6a_mathematics","participant":{"type":"class","id":"class_6a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_russian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_language","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_belarusian_literature","participant":{"type":"class","id":"class_6a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_english","participant":{"type":"class","id":"class_6a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_physical_education","participant":{"type":"class","id":"class_6a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_technology","participant":{"type":"class","id":"class_6a"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_informatics","participant":{"type":"class","id":"class_6a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_art","participant":{"type":"class","id":"class_6a"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_biology","participant":{"type":"class","id":"class_6a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_geography","participant":{"type":"class","id":"class_6a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_history_belarus","participant":{"type":"class","id":"class_6a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6a_world_history","participant":{"type":"class","id":"class_6a"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6a"]},{"id":"req_6b_mathematics","participant":{"type":"class","id":"class_6b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_russian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_language","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_belarusian_literature","participant":{"type":"class","id":"class_6b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_english","participant":{"type":"class","id":"class_6b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_physical_education","participant":{"type":"class","id":"class_6b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_technology","participant":{"type":"class","id":"class_6b"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_informatics","participant":{"type":"class","id":"class_6b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_art","participant":{"type":"class","id":"class_6b"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_biology","participant":{"type":"class","id":"class_6b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_geography","participant":{"type":"class","id":"class_6b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_history_belarus","participant":{"type":"class","id":"class_6b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6b_world_history","participant":{"type":"class","id":"class_6b"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6b"]},{"id":"req_6v_mathematics","participant":{"type":"class","id":"class_6v"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_russian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_language","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_belarusian_literature","participant":{"type":"class","id":"class_6v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_english","participant":{"type":"class","id":"class_6v"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_physical_education","participant":{"type":"class","id":"class_6v"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_technology","participant":{"type":"class","id":"class_6v"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_informatics","participant":{"type":"class","id":"class_6v"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_art","participant":{"type":"class","id":"class_6v"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_biology","participant":{"type":"class","id":"class_6v"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_geography","participant":{"type":"class","id":"class_6v"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_history_belarus","participant":{"type":"class","id":"class_6v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_6v_world_history","participant":{"type":"class","id":"class_6v"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_6v"]},{"id":"req_7a_math","participant":{"type":"class","id":"class_7a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_russian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_language","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_belarusian_literature","participant":{"type":"class","id":"class_7a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_en_1","participant":{"type":"class","id":"class_7a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physical_education","participant":{"type":"class","id":"class_7a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_technology","participant":{"type":"class","id":"class_7a"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_informatics","participant":{"type":"class","id":"class_7a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_joint_advisory","participant":{"type":"class","id":"class_7a"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_biology","participant":{"type":"class","id":"class_7a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_geography","participant":{"type":"class","id":"class_7a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_history_belarus","participant":{"type":"class","id":"class_7a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_world_history","participant":{"type":"class","id":"class_7a"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_physics","participant":{"type":"class","id":"class_7a"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7a_chemistry","participant":{"type":"class","id":"class_7a"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7a"]},{"id":"req_7b_mathematics","participant":{"type":"class","id":"class_7b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_russian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_language","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_belarusian_literature","participant":{"type":"class","id":"class_7b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_english","participant":{"type":"class","id":"class_7b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physical_education","participant":{"type":"class","id":"class_7b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_technology","participant":{"type":"class","id":"class_7b"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_informatics","participant":{"type":"class","id":"class_7b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_art","participant":{"type":"class","id":"class_7b"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_biology","participant":{"type":"class","id":"class_7b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_geography","participant":{"type":"class","id":"class_7b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_history_belarus","participant":{"type":"class","id":"class_7b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_world_history","participant":{"type":"class","id":"class_7b"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_physics","participant":{"type":"class","id":"class_7b"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7b_chemistry","participant":{"type":"class","id":"class_7b"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7b"]},{"id":"req_7v_mathematics","participant":{"type":"class","id":"class_7v"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_russian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_language","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_belarusian_literature","participant":{"type":"class","id":"class_7v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_english","participant":{"type":"class","id":"class_7v"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physical_education","participant":{"type":"class","id":"class_7v"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_technology","participant":{"type":"class","id":"class_7v"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_informatics","participant":{"type":"class","id":"class_7v"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_art","participant":{"type":"class","id":"class_7v"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_biology","participant":{"type":"class","id":"class_7v"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_geography","participant":{"type":"class","id":"class_7v"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_history_belarus","participant":{"type":"class","id":"class_7v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_world_history","participant":{"type":"class","id":"class_7v"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_physics","participant":{"type":"class","id":"class_7v"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_7v_chemistry","participant":{"type":"class","id":"class_7v"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_7v"]},{"id":"req_8a_mathematics","participant":{"type":"class","id":"class_8a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_russian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_language","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_belarusian_literature","participant":{"type":"class","id":"class_8a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_english","participant":{"type":"class","id":"class_8a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physical_education","participant":{"type":"class","id":"class_8a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_technology","participant":{"type":"class","id":"class_8a"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_informatics","participant":{"type":"class","id":"class_8a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_art","participant":{"type":"class","id":"class_8a"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_biology","participant":{"type":"class","id":"class_8a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_geography","participant":{"type":"class","id":"class_8a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_history_belarus","participant":{"type":"class","id":"class_8a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_world_history","participant":{"type":"class","id":"class_8a"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_physics","participant":{"type":"class","id":"class_8a"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8a_chemistry","participant":{"type":"class","id":"class_8a"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":2,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8a"]},{"id":"req_8b_mathematics","participant":{"type":"class","id":"class_8b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_russian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_language","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_belarusian_literature","participant":{"type":"class","id":"class_8b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_english","participant":{"type":"class","id":"class_8b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physical_education","participant":{"type":"class","id":"class_8b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_technology","participant":{"type":"class","id":"class_8b"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_informatics","participant":{"type":"class","id":"class_8b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_art","participant":{"type":"class","id":"class_8b"},"subject_id":"art","eligible_teacher_ids":["t_art","t_art_2","t_art_3","t_art_4"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_biology","participant":{"type":"class","id":"class_8b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_geography","participant":{"type":"class","id":"class_8b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_history_belarus","participant":{"type":"class","id":"class_8b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_world_history","participant":{"type":"class","id":"class_8b"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_physics","participant":{"type":"class","id":"class_8b"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_8b_chemistry","participant":{"type":"class","id":"class_8b"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_8b"]},{"id":"req_9a_mathematics","participant":{"type":"class","id":"class_9a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_russian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_language","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_belarusian_literature","participant":{"type":"class","id":"class_9a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_english","participant":{"type":"class","id":"class_9a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physical_education","participant":{"type":"class","id":"class_9a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_technology","participant":{"type":"class","id":"class_9a"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_informatics","participant":{"type":"class","id":"class_9a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_biology","participant":{"type":"class","id":"class_9a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_geography","participant":{"type":"class","id":"class_9a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_history_belarus","participant":{"type":"class","id":"class_9a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_world_history","participant":{"type":"class","id":"class_9a"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_physics","participant":{"type":"class","id":"class_9a"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_chemistry","participant":{"type":"class","id":"class_9a"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9a_social_studies","participant":{"type":"class","id":"class_9a"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9a"]},{"id":"req_9b_mathematics","participant":{"type":"class","id":"class_9b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_russian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_language","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_belarusian_literature","participant":{"type":"class","id":"class_9b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_english","participant":{"type":"class","id":"class_9b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physical_education","participant":{"type":"class","id":"class_9b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_technology","participant":{"type":"class","id":"class_9b"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_informatics","participant":{"type":"class","id":"class_9b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_biology","participant":{"type":"class","id":"class_9b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_geography","participant":{"type":"class","id":"class_9b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_history_belarus","participant":{"type":"class","id":"class_9b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_world_history","participant":{"type":"class","id":"class_9b"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_physics","participant":{"type":"class","id":"class_9b"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_chemistry","participant":{"type":"class","id":"class_9b"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9b_social_studies","participant":{"type":"class","id":"class_9b"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9b"]},{"id":"req_9v_mathematics","participant":{"type":"class","id":"class_9v"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_russian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_language","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_belarusian_literature","participant":{"type":"class","id":"class_9v"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_english","participant":{"type":"class","id":"class_9v"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":5,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physical_education","participant":{"type":"class","id":"class_9v"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_technology","participant":{"type":"class","id":"class_9v"},"subject_id":"technology","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_informatics","participant":{"type":"class","id":"class_9v"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_biology","participant":{"type":"class","id":"class_9v"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_geography","participant":{"type":"class","id":"class_9v"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_history_belarus","participant":{"type":"class","id":"class_9v"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_world_history","participant":{"type":"class","id":"class_9v"},"subject_id":"world_history","eligible_teacher_ids":["t_world_history","t_world_history_2","t_world_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_physics","participant":{"type":"class","id":"class_9v"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_chemistry","participant":{"type":"class","id":"class_9v"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_9v_social_studies","participant":{"type":"class","id":"class_9v"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_9v"]},{"id":"req_10a_mathematics","participant":{"type":"class","id":"class_10a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physics","participant":{"type":"class","id":"class_10a"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_chemistry","participant":{"type":"class","id":"class_10a"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_biology","participant":{"type":"class","id":"class_10a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_russian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_language","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_belarusian_literature","participant":{"type":"class","id":"class_10a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_english","participant":{"type":"class","id":"class_10a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_physical_education","participant":{"type":"class","id":"class_10a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_informatics","participant":{"type":"class","id":"class_10a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_geography","participant":{"type":"class","id":"class_10a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_history_belarus","participant":{"type":"class","id":"class_10a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_social_studies","participant":{"type":"class","id":"class_10a"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_technical_drawing","participant":{"type":"class","id":"class_10a"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10a_defense_medical","participant":{"type":"class","id":"class_10a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_defense"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10a"]},{"id":"req_10b_mathematics","participant":{"type":"class","id":"class_10b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physics","participant":{"type":"class","id":"class_10b"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_chemistry","participant":{"type":"class","id":"class_10b"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_biology","participant":{"type":"class","id":"class_10b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_russian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_language","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_belarusian_literature","participant":{"type":"class","id":"class_10b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_english","participant":{"type":"class","id":"class_10b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_physical_education","participant":{"type":"class","id":"class_10b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_informatics","participant":{"type":"class","id":"class_10b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_geography","participant":{"type":"class","id":"class_10b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_history_belarus","participant":{"type":"class","id":"class_10b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_social_studies","participant":{"type":"class","id":"class_10b"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_technical_drawing","participant":{"type":"class","id":"class_10b"},"subject_id":"technical_drawing","eligible_teacher_ids":["t_technology","t_technology_2","t_technology_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_10b_defense_medical","participant":{"type":"class","id":"class_10b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_defense"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_10b"]},{"id":"req_11a_mathematics","participant":{"type":"class","id":"class_11a"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physics","participant":{"type":"class","id":"class_11a"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_chemistry","participant":{"type":"class","id":"class_11a"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_biology","participant":{"type":"class","id":"class_11a"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_russian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_language","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_belarusian_literature","participant":{"type":"class","id":"class_11a"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_english","participant":{"type":"class","id":"class_11a"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_physical_education","participant":{"type":"class","id":"class_11a"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_informatics","participant":{"type":"class","id":"class_11a"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_geography","participant":{"type":"class","id":"class_11a"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_history_belarus","participant":{"type":"class","id":"class_11a"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_social_studies","participant":{"type":"class","id":"class_11a"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_astronomy","participant":{"type":"class","id":"class_11a"},"subject_id":"astronomy","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11a_defense_medical","participant":{"type":"class","id":"class_11a"},"subject_id":"defense_medical","eligible_teacher_ids":["t_defense"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11a"]},{"id":"req_11b_mathematics","participant":{"type":"class","id":"class_11b"},"subject_id":"mathematics","eligible_teacher_ids":["t_math","t_math_2","t_math_3","t_math_4","t_math_5","t_math_6","t_math_7"],"weekly_lessons":6,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physics","participant":{"type":"class","id":"class_11b"},"subject_id":"physics","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_chemistry","participant":{"type":"class","id":"class_11b"},"subject_id":"chemistry","eligible_teacher_ids":["t_chemistry","t_chemistry_2"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_biology","participant":{"type":"class","id":"class_11b"},"subject_id":"biology","eligible_teacher_ids":["t_biology","t_biology_2","t_biology_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_language","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_russian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"russian_literature","eligible_teacher_ids":["t_russian_1","t_russian_2","t_russian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_language","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_language","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_belarusian_literature","participant":{"type":"class","id":"class_11b"},"subject_id":"belarusian_literature","eligible_teacher_ids":["t_belarusian_1","t_belarusian_2","t_belarusian_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_english","participant":{"type":"class","id":"class_11b"},"subject_id":"english","eligible_teacher_ids":["t_english_1","t_english_2","t_english_3","t_english_4","t_english_5","t_english_6"],"weekly_lessons":4,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_physical_education","participant":{"type":"class","id":"class_11b"},"subject_id":"physical_education","eligible_teacher_ids":["t_pe_1","t_pe_2","t_pe_3","t_pe_4","t_pe_5"],"weekly_lessons":3,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_informatics","participant":{"type":"class","id":"class_11b"},"subject_id":"informatics","eligible_teacher_ids":["t_informatics","t_informatics_2","t_informatics_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_geography","participant":{"type":"class","id":"class_11b"},"subject_id":"geography","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_history_belarus","participant":{"type":"class","id":"class_11b"},"subject_id":"history_belarus","eligible_teacher_ids":["t_belarus_history","t_belarus_history_2","t_belarus_history_3"],"weekly_lessons":2,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_social_studies","participant":{"type":"class","id":"class_11b"},"subject_id":"social_studies","eligible_teacher_ids":["t_geography","t_geography_2","t_geography_3"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_astronomy","participant":{"type":"class","id":"class_11b"},"subject_id":"astronomy","eligible_teacher_ids":["t_physics","t_physics_2"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]},{"id":"req_11b_defense_medical","participant":{"type":"class","id":"class_11b"},"subject_id":"defense_medical","eligible_teacher_ids":["t_defense"],"weekly_lessons":1,"block_length":1,"required_room_capabilities":["general"],"allowed_classroom_ids":["room_11b"]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
-      <x:c r="A14" s="16" t="str">
+      <x:c r="A14" s="17" t="str">
         <x:v>resource_availability</x:v>
       </x:c>
-      <x:c r="B14" s="15" t="str">
-        <x:v>[{"resource":{"type":"class","id":"class_5a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9v"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"teacher","id":"t_math"},"unavailable_slots":[],"preferred_slots":[]},{"resource":{"type":"teacher","id":"t_7a"},"unavailable_slots":[],"preferred_slots":[]},{"resource":{"type":"classroom","id":"science_lab"},"unavailable_slots":[{"day_id":"fri","period_id":"p6"}],"preferred_slots":[]}]</x:v>
+      <x:c r="B14" s="16" t="str">
+        <x:v>[{"resource":{"type":"class","id":"class_5a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_5v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p6"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_6v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7a"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7b"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_7v"},"unavailable_slots":[{"day_id":"mon","period_id":"p7"},{"day_id":"tue","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_8b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9a"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9b"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_9v"},"unavailable_slots":[{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_10b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11a"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"class","id":"class_11b"},"unavailable_slots":[{"day_id":"wed","period_id":"p7"},{"day_id":"thu","period_id":"p7"},{"day_id":"fri","period_id":"p7"}],"preferred_slots":[]},{"resource":{"type":"teacher","id":"t_defense"},"unavailable_slots":[],"preferred_slots":[]}]</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
-      <x:c r="A15" s="16" t="str">
+      <x:c r="A15" s="17" t="str">
         <x:v>fixed_lessons</x:v>
       </x:c>
-      <x:c r="B15" s="15" t="str">
-        <x:v>[{"id":"fixed_joint_advisory","requirement_id":"req_joint_advisory","occurrence_index":0,"slot":{"day_id":"mon","period_id":"p1"},"teacher_id":"t_7a","classroom_id":"room_7a"}]</x:v>
+      <x:c r="B15" s="16" t="str">
+        <x:v>[{"id":"fixed_joint_advisory","requirement_id":"req_joint_advisory","occurrence_index":0,"slot":{"day_id":"mon","period_id":"p1"},"teacher_id":"t_art","classroom_id":"room_7a"}]</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
-      <x:c r="A16" s="16" t="str">
+      <x:c r="A16" s="17" t="str">
         <x:v>policies</x:v>
       </x:c>
-      <x:c r="B16" s="15" t="str">
-        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_5a"},"maximum":6},{"resource":{"type":"teacher","id":"t_math"},"maximum":6},{"resource":{"type":"class","id":"class_5b"},"maximum":6},{"resource":{"type":"teacher","id":"t_5b"},"maximum":6},{"resource":{"type":"class","id":"class_5v"},"maximum":6},{"resource":{"type":"teacher","id":"t_5v"},"maximum":6},{"resource":{"type":"class","id":"class_6a"},"maximum":6},{"resource":{"type":"teacher","id":"t_6a"},"maximum":6},{"resource":{"type":"class","id":"class_6b"},"maximum":6},{"resource":{"type":"teacher","id":"t_6b"},"maximum":6},{"resource":{"type":"class","id":"class_6v"},"maximum":6},{"resource":{"type":"teacher","id":"t_6v"},"maximum":6},{"resource":{"type":"class","id":"class_7a"},"maximum":7},{"resource":{"type":"teacher","id":"t_7a"},"maximum":7},{"resource":{"type":"class","id":"class_7b"},"maximum":7},{"resource":{"type":"teacher","id":"t_7b"},"maximum":7},{"resource":{"type":"class","id":"class_7v"},"maximum":7},{"resource":{"type":"teacher","id":"t_7v"},"maximum":7},{"resource":{"type":"class","id":"class_8a"},"maximum":7},{"resource":{"type":"teacher","id":"t_8a"},"maximum":7},{"resource":{"type":"class","id":"class_8b"},"maximum":7},{"resource":{"type":"teacher","id":"t_8b"},"maximum":7},{"resource":{"type":"class","id":"class_9a"},"maximum":7},{"resource":{"type":"teacher","id":"t_9a"},"maximum":7},{"resource":{"type":"class","id":"class_9b"},"maximum":7},{"resource":{"type":"teacher","id":"t_9b"},"maximum":7},{"resource":{"type":"class","id":"class_9v"},"maximum":7},{"resource":{"type":"teacher","id":"t_9v"},"maximum":7},{"resource":{"type":"class","id":"class_10a"},"maximum":7},{"resource":{"type":"teacher","id":"t_10a"},"maximum":7},{"resource":{"type":"class","id":"class_10b"},"maximum":7},{"resource":{"type":"teacher","id":"t_10b"},"maximum":7},{"resource":{"type":"class","id":"class_11a"},"maximum":7},{"resource":{"type":"teacher","id":"t_11a"},"maximum":7},{"resource":{"type":"class","id":"class_11b"},"maximum":7},{"resource":{"type":"teacher","id":"t_11b"},"maximum":7}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_5a"},"target":11},{"participant":{"type":"class","id":"class_5b"},"target":11},{"participant":{"type":"class","id":"class_5v"},"target":11},{"participant":{"type":"class","id":"class_6a"},"target":11},{"participant":{"type":"class","id":"class_6b"},"target":11},{"participant":{"type":"class","id":"class_6v"},"target":11},{"participant":{"type":"class","id":"class_7a"},"target":13},{"participant":{"type":"class","id":"class_7b"},"target":13},{"participant":{"type":"class","id":"class_7v"},"target":13},{"participant":{"type":"class","id":"class_8a"},"target":13},{"participant":{"type":"class","id":"class_8b"},"target":13},{"participant":{"type":"class","id":"class_9a"},"target":13},{"participant":{"type":"class","id":"class_9b"},"target":13},{"participant":{"type":"class","id":"class_9v"},"target":13},{"participant":{"type":"class","id":"class_10a"},"target":13},{"participant":{"type":"class","id":"class_10b"},"target":13},{"participant":{"type":"class","id":"class_11a"},"target":13},{"participant":{"type":"class","id":"class_11b"},"target":13}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P1","weight":40},{"constraint_id":"SC-003","priority":"P1","weight":200},{"constraint_id":"SC-004","priority":"P2","weight":3},{"constraint_id":"SC-005","priority":"P2","weight":4}]}</x:v>
+      <x:c r="B16" s="16" t="str">
+        <x:v>{"daily_limits":[{"resource":{"type":"class","id":"class_5a"},"maximum":6},{"resource":{"type":"class","id":"class_5b"},"maximum":6},{"resource":{"type":"class","id":"class_5v"},"maximum":6},{"resource":{"type":"class","id":"class_6a"},"maximum":6},{"resource":{"type":"class","id":"class_6b"},"maximum":6},{"resource":{"type":"class","id":"class_6v"},"maximum":6},{"resource":{"type":"class","id":"class_7a"},"maximum":7},{"resource":{"type":"class","id":"class_7b"},"maximum":7},{"resource":{"type":"class","id":"class_7v"},"maximum":7},{"resource":{"type":"class","id":"class_8a"},"maximum":7},{"resource":{"type":"class","id":"class_8b"},"maximum":7},{"resource":{"type":"class","id":"class_9a"},"maximum":7},{"resource":{"type":"class","id":"class_9b"},"maximum":7},{"resource":{"type":"class","id":"class_9v"},"maximum":7},{"resource":{"type":"class","id":"class_10a"},"maximum":7},{"resource":{"type":"class","id":"class_10b"},"maximum":7},{"resource":{"type":"class","id":"class_11a"},"maximum":7},{"resource":{"type":"class","id":"class_11b"},"maximum":7},{"resource":{"type":"teacher","id":"t_math"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_4"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_5"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_6"},"maximum":7},{"resource":{"type":"teacher","id":"t_math_7"},"maximum":7},{"resource":{"type":"teacher","id":"t_russian_1"},"maximum":7},{"resource":{"type":"teacher","id":"t_russian_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_russian_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarusian_1"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarusian_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarusian_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_1"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_4"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_5"},"maximum":7},{"resource":{"type":"teacher","id":"t_english_6"},"maximum":7},{"resource":{"type":"teacher","id":"t_pe_1"},"maximum":7},{"resource":{"type":"teacher","id":"t_pe_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_pe_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_pe_4"},"maximum":7},{"resource":{"type":"teacher","id":"t_pe_5"},"maximum":7},{"resource":{"type":"teacher","id":"t_physics"},"maximum":7},{"resource":{"type":"teacher","id":"t_physics_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_chemistry"},"maximum":7},{"resource":{"type":"teacher","id":"t_chemistry_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_biology"},"maximum":7},{"resource":{"type":"teacher","id":"t_biology_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_biology_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarus_history"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarus_history_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_belarus_history_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_world_history"},"maximum":7},{"resource":{"type":"teacher","id":"t_world_history_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_world_history_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_geography"},"maximum":7},{"resource":{"type":"teacher","id":"t_geography_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_geography_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_technology"},"maximum":7},{"resource":{"type":"teacher","id":"t_technology_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_technology_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_art"},"maximum":7},{"resource":{"type":"teacher","id":"t_art_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_art_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_art_4"},"maximum":7},{"resource":{"type":"teacher","id":"t_informatics"},"maximum":7},{"resource":{"type":"teacher","id":"t_informatics_2"},"maximum":7},{"resource":{"type":"teacher","id":"t_informatics_3"},"maximum":7},{"resource":{"type":"teacher","id":"t_defense"},"maximum":7}],"difficult_load_targets":[{"participant":{"type":"class","id":"class_5a"},"target":11},{"participant":{"type":"class","id":"class_5b"},"target":11},{"participant":{"type":"class","id":"class_5v"},"target":11},{"participant":{"type":"class","id":"class_6a"},"target":11},{"participant":{"type":"class","id":"class_6b"},"target":11},{"participant":{"type":"class","id":"class_6v"},"target":11},{"participant":{"type":"class","id":"class_7a"},"target":13},{"participant":{"type":"class","id":"class_7b"},"target":13},{"participant":{"type":"class","id":"class_7v"},"target":13},{"participant":{"type":"class","id":"class_8a"},"target":13},{"participant":{"type":"class","id":"class_8b"},"target":13},{"participant":{"type":"class","id":"class_9a"},"target":13},{"participant":{"type":"class","id":"class_9b"},"target":13},{"participant":{"type":"class","id":"class_9v"},"target":13},{"participant":{"type":"class","id":"class_10a"},"target":13},{"participant":{"type":"class","id":"class_10b"},"target":13},{"participant":{"type":"class","id":"class_11a"},"target":13},{"participant":{"type":"class","id":"class_11b"},"target":13}],"soft_constraint_weights":[{"constraint_id":"SC-001","priority":"P1","weight":10},{"constraint_id":"SC-002","priority":"P1","weight":40},{"constraint_id":"SC-003","priority":"P1","weight":200},{"constraint_id":"SC-004","priority":"P2","weight":10},{"constraint_id":"SC-005","priority":"P2","weight":30},{"constraint_id":"SC-019","priority":"P2","weight":30}]}</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
-      <x:c r="A17" s="16" t="str">
+      <x:c r="A17" s="17" t="str">
         <x:v>timetable_versions</x:v>
       </x:c>
-      <x:c r="B17" s="15" t="str">
+      <x:c r="B17" s="16" t="str">
         <x:v>[]</x:v>
       </x:c>
     </x:row>

</xml_diff>